<commit_message>
payments service and music table schema
</commit_message>
<xml_diff>
--- a/DBMS Game Store Docs/User Stories.xlsx
+++ b/DBMS Game Store Docs/User Stories.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryanc\Desktop\final_year_project\DBMS Game Store Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FED3ADA7-39FB-4D96-94F1-7D34F56EF3A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1997A2F9-BB7A-48F5-91BF-D015654D870B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{91133E6D-6CC4-4AFD-BF36-5C9837FF4593}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="235" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="264">
   <si>
     <t>As a admin,</t>
   </si>
@@ -332,12 +332,6 @@
     <t>I want to view my purchases,</t>
   </si>
   <si>
-    <t>Verify purchased PS4 game is displayed to the customer.</t>
-  </si>
-  <si>
-    <t>Verify purchased Xbox game is displayed to the customer.</t>
-  </si>
-  <si>
     <t>so I can calculate sales.</t>
   </si>
   <si>
@@ -563,9 +557,6 @@
     <t>Verify order number is displayed.</t>
   </si>
   <si>
-    <t>Verify customer identifier number is displayed.</t>
-  </si>
-  <si>
     <t>so I can let different accounts see different info.</t>
   </si>
   <si>
@@ -624,6 +615,219 @@
   </si>
   <si>
     <t>so I can remove unnecessary details.</t>
+  </si>
+  <si>
+    <t>so I can let customers buy games and music.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is created for music.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is created for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is created for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is created for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is created for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is created for music.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is created for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is created for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is created for music.</t>
+  </si>
+  <si>
+    <t>I want to read paymets,</t>
+  </si>
+  <si>
+    <t>I want to delete payments,</t>
+  </si>
+  <si>
+    <t>I want to update payments,</t>
+  </si>
+  <si>
+    <t>I want to create payments,</t>
+  </si>
+  <si>
+    <t>Verify order id is read for payments.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is read for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is read for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is read for music.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is read for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is read for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is read for music.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is read for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is read for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is read for music.</t>
+  </si>
+  <si>
+    <t>Verify order id is updated for payments.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is updated for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is updated for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is updated for music.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is updated for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is updated for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is updated for music.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is updated for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is updated for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is updated for music.</t>
+  </si>
+  <si>
+    <t>Verify order id is deleted for payments.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is deleted for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is deleted for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment amount is deleted for music.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is deleted for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is deleted for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is deleted for music.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is deleted for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is deleted for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is deleted for music.</t>
+  </si>
+  <si>
+    <t>so I can ensure payment confirmation.</t>
+  </si>
+  <si>
+    <t>so I can change payment status.</t>
+  </si>
+  <si>
+    <t>so I can remove uneeded payment information.</t>
+  </si>
+  <si>
+    <t>Verify order id is created for payment.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is read for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is read for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment cost is read for music.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is updated for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is updated for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment cost is updated for music.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is deleted for PS4 games.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is deleted for Xbox games.</t>
+  </si>
+  <si>
+    <t>Verfiy payment cost is deleted for music.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is created for PS4 games 0&gt; &amp; &lt;$69.99.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is created for Xbox games 0&gt; &amp; &lt;$69.99.</t>
+  </si>
+  <si>
+    <t>Verfiy payment cost is created for music 0&gt; &amp; &lt;$5.00.</t>
+  </si>
+  <si>
+    <t>Verify album title is created 0&gt; &amp; &lt;10.</t>
+  </si>
+  <si>
+    <t>Verify music title is read.</t>
+  </si>
+  <si>
+    <t>Verify music title is updated.</t>
+  </si>
+  <si>
+    <t>Verify music title is deleted.</t>
+  </si>
+  <si>
+    <t>Verify album price is created 0&gt; &amp;  $5.00.</t>
+  </si>
+  <si>
+    <t>Verify album price is read.</t>
+  </si>
+  <si>
+    <t>Verify album price is updated.</t>
+  </si>
+  <si>
+    <t>Verify album price is deleted.</t>
+  </si>
+  <si>
+    <t>Verify purchased PS4 game title is displayed to the customer.</t>
+  </si>
+  <si>
+    <t>Verify purchased Xbox game title is displayed to the customer.</t>
+  </si>
+  <si>
+    <t>Verify platform type is displayed to the customer.</t>
   </si>
 </sst>
 </file>
@@ -719,7 +923,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -731,6 +935,7 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1065,7 +1270,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62F77FC3-F402-4BE8-8A68-6767566B15A6}">
-  <dimension ref="A1:K183"/>
+  <dimension ref="A1:K247"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1077,7 +1282,7 @@
       <c r="D1" s="10"/>
       <c r="E1" s="10"/>
       <c r="F1" s="10" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="G1" s="10"/>
       <c r="H1" s="10"/>
@@ -1087,14 +1292,14 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
       <c r="E2" s="10"/>
       <c r="F2" s="10" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
@@ -1104,14 +1309,14 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="10"/>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
       <c r="F3" s="10" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="10"/>
@@ -1154,7 +1359,7 @@
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="G6" s="10"/>
       <c r="H6" s="10"/>
@@ -1164,14 +1369,14 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="10"/>
@@ -1181,14 +1386,14 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="G8" s="10"/>
       <c r="H8" s="10"/>
@@ -1231,7 +1436,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="G11" s="10"/>
       <c r="H11" s="10"/>
@@ -1241,14 +1446,14 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
@@ -1258,14 +1463,14 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="G13" s="10"/>
       <c r="H13" s="10"/>
@@ -1308,7 +1513,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
@@ -1318,14 +1523,14 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
@@ -1335,14 +1540,14 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
@@ -2281,7 +2486,7 @@
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="G85" s="3"/>
       <c r="H85" s="3"/>
@@ -2298,7 +2503,7 @@
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="G86" s="3"/>
       <c r="H86" s="3"/>
@@ -2315,7 +2520,7 @@
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="G87" s="3"/>
       <c r="H87" s="3"/>
@@ -2330,7 +2535,7 @@
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="G88" s="3"/>
       <c r="H88" s="3"/>
@@ -2345,7 +2550,7 @@
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="G89" s="3"/>
       <c r="H89" s="3"/>
@@ -2360,7 +2565,7 @@
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="G90" s="3"/>
       <c r="H90" s="3"/>
@@ -2375,7 +2580,7 @@
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G91" s="3"/>
       <c r="H91" s="3"/>
@@ -2390,7 +2595,7 @@
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3" t="s">
-        <v>140</v>
+        <v>253</v>
       </c>
       <c r="G92" s="3"/>
       <c r="H92" s="3"/>
@@ -2405,7 +2610,7 @@
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3" t="s">
-        <v>154</v>
+        <v>138</v>
       </c>
       <c r="G93" s="3"/>
       <c r="H93" s="3"/>
@@ -2420,7 +2625,7 @@
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="G94" s="3"/>
       <c r="H94" s="3"/>
@@ -2434,7 +2639,9 @@
       <c r="C95" s="3"/>
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
-      <c r="F95" s="3"/>
+      <c r="F95" s="3" t="s">
+        <v>257</v>
+      </c>
       <c r="G95" s="3"/>
       <c r="H95" s="3"/>
       <c r="I95" s="3"/>
@@ -2442,15 +2649,13 @@
       <c r="K95" s="3"/>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A96" s="3" t="s">
-        <v>95</v>
-      </c>
+      <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3" t="s">
-        <v>126</v>
+        <v>139</v>
       </c>
       <c r="G96" s="3"/>
       <c r="H96" s="3"/>
@@ -2459,16 +2664,12 @@
       <c r="K96" s="3"/>
     </row>
     <row r="97" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A97" s="3" t="s">
-        <v>72</v>
-      </c>
+      <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
-      <c r="F97" s="3" t="s">
-        <v>121</v>
-      </c>
+      <c r="F97" s="3"/>
       <c r="G97" s="3"/>
       <c r="H97" s="3"/>
       <c r="I97" s="3"/>
@@ -2477,14 +2678,14 @@
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="G98" s="3"/>
       <c r="H98" s="3"/>
@@ -2493,13 +2694,15 @@
       <c r="K98" s="3"/>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A99" s="3"/>
+      <c r="A99" s="3" t="s">
+        <v>72</v>
+      </c>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="G99" s="3"/>
       <c r="H99" s="3"/>
@@ -2508,13 +2711,15 @@
       <c r="K99" s="3"/>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A100" s="3"/>
+      <c r="A100" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
       <c r="G100" s="3"/>
       <c r="H100" s="3"/>
@@ -2529,7 +2734,7 @@
       <c r="D101" s="3"/>
       <c r="E101" s="3"/>
       <c r="F101" s="3" t="s">
-        <v>142</v>
+        <v>126</v>
       </c>
       <c r="G101" s="3"/>
       <c r="H101" s="3"/>
@@ -2544,7 +2749,7 @@
       <c r="D102" s="3"/>
       <c r="E102" s="3"/>
       <c r="F102" s="3" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="G102" s="3"/>
       <c r="H102" s="3"/>
@@ -2559,7 +2764,7 @@
       <c r="D103" s="3"/>
       <c r="E103" s="3"/>
       <c r="F103" s="3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="G103" s="3"/>
       <c r="H103" s="3"/>
@@ -2574,7 +2779,7 @@
       <c r="D104" s="3"/>
       <c r="E104" s="3"/>
       <c r="F104" s="3" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="G104" s="3"/>
       <c r="H104" s="3"/>
@@ -2589,7 +2794,7 @@
       <c r="D105" s="3"/>
       <c r="E105" s="3"/>
       <c r="F105" s="3" t="s">
-        <v>145</v>
+        <v>254</v>
       </c>
       <c r="G105" s="3"/>
       <c r="H105" s="3"/>
@@ -2603,7 +2808,9 @@
       <c r="C106" s="3"/>
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
-      <c r="F106" s="3"/>
+      <c r="F106" s="3" t="s">
+        <v>142</v>
+      </c>
       <c r="G106" s="3"/>
       <c r="H106" s="3"/>
       <c r="I106" s="3"/>
@@ -2611,15 +2818,13 @@
       <c r="K106" s="3"/>
     </row>
     <row r="107" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A107" s="3" t="s">
-        <v>95</v>
-      </c>
+      <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
       <c r="D107" s="3"/>
       <c r="E107" s="3"/>
       <c r="F107" s="3" t="s">
-        <v>129</v>
+        <v>154</v>
       </c>
       <c r="G107" s="3"/>
       <c r="H107" s="3"/>
@@ -2628,15 +2833,13 @@
       <c r="K107" s="3"/>
     </row>
     <row r="108" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A108" s="3" t="s">
-        <v>73</v>
-      </c>
+      <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
       <c r="D108" s="3"/>
       <c r="E108" s="3"/>
       <c r="F108" s="3" t="s">
-        <v>122</v>
+        <v>258</v>
       </c>
       <c r="G108" s="3"/>
       <c r="H108" s="3"/>
@@ -2645,15 +2848,13 @@
       <c r="K108" s="3"/>
     </row>
     <row r="109" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A109" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="A109" s="3"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
       <c r="D109" s="3"/>
       <c r="E109" s="3"/>
       <c r="F109" s="3" t="s">
-        <v>130</v>
+        <v>143</v>
       </c>
       <c r="G109" s="3"/>
       <c r="H109" s="3"/>
@@ -2667,9 +2868,7 @@
       <c r="C110" s="3"/>
       <c r="D110" s="3"/>
       <c r="E110" s="3"/>
-      <c r="F110" s="3" t="s">
-        <v>131</v>
-      </c>
+      <c r="F110" s="3"/>
       <c r="G110" s="3"/>
       <c r="H110" s="3"/>
       <c r="I110" s="3"/>
@@ -2677,13 +2876,15 @@
       <c r="K110" s="3"/>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A111" s="3"/>
+      <c r="A111" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
       <c r="E111" s="3"/>
       <c r="F111" s="3" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="G111" s="3"/>
       <c r="H111" s="3"/>
@@ -2692,13 +2893,15 @@
       <c r="K111" s="3"/>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A112" s="3"/>
+      <c r="A112" s="3" t="s">
+        <v>73</v>
+      </c>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
       <c r="E112" s="3"/>
       <c r="F112" s="3" t="s">
-        <v>146</v>
+        <v>120</v>
       </c>
       <c r="G112" s="3"/>
       <c r="H112" s="3"/>
@@ -2707,13 +2910,15 @@
       <c r="K112" s="3"/>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A113" s="3"/>
+      <c r="A113" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
       <c r="D113" s="3"/>
       <c r="E113" s="3"/>
       <c r="F113" s="3" t="s">
-        <v>147</v>
+        <v>128</v>
       </c>
       <c r="G113" s="3"/>
       <c r="H113" s="3"/>
@@ -2728,7 +2933,7 @@
       <c r="D114" s="3"/>
       <c r="E114" s="3"/>
       <c r="F114" s="3" t="s">
-        <v>148</v>
+        <v>129</v>
       </c>
       <c r="G114" s="3"/>
       <c r="H114" s="3"/>
@@ -2743,7 +2948,7 @@
       <c r="D115" s="3"/>
       <c r="E115" s="3"/>
       <c r="F115" s="3" t="s">
-        <v>157</v>
+        <v>135</v>
       </c>
       <c r="G115" s="3"/>
       <c r="H115" s="3"/>
@@ -2758,7 +2963,7 @@
       <c r="D116" s="3"/>
       <c r="E116" s="3"/>
       <c r="F116" s="3" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="G116" s="3"/>
       <c r="H116" s="3"/>
@@ -2772,7 +2977,9 @@
       <c r="C117" s="3"/>
       <c r="D117" s="3"/>
       <c r="E117" s="3"/>
-      <c r="F117" s="3"/>
+      <c r="F117" s="3" t="s">
+        <v>145</v>
+      </c>
       <c r="G117" s="3"/>
       <c r="H117" s="3"/>
       <c r="I117" s="3"/>
@@ -2780,15 +2987,13 @@
       <c r="K117" s="3"/>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A118" s="3" t="s">
-        <v>95</v>
-      </c>
+      <c r="A118" s="3"/>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
       <c r="E118" s="3"/>
       <c r="F118" s="3" t="s">
-        <v>132</v>
+        <v>255</v>
       </c>
       <c r="G118" s="3"/>
       <c r="H118" s="3"/>
@@ -2797,15 +3002,13 @@
       <c r="K118" s="3"/>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A119" s="3" t="s">
-        <v>74</v>
-      </c>
+      <c r="A119" s="3"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
       <c r="D119" s="3"/>
       <c r="E119" s="3"/>
       <c r="F119" s="3" t="s">
-        <v>123</v>
+        <v>146</v>
       </c>
       <c r="G119" s="3"/>
       <c r="H119" s="3"/>
@@ -2814,15 +3017,13 @@
       <c r="K119" s="3"/>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A120" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="A120" s="3"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
       <c r="D120" s="3"/>
       <c r="E120" s="3"/>
       <c r="F120" s="3" t="s">
-        <v>133</v>
+        <v>155</v>
       </c>
       <c r="G120" s="3"/>
       <c r="H120" s="3"/>
@@ -2837,7 +3038,7 @@
       <c r="D121" s="3"/>
       <c r="E121" s="3"/>
       <c r="F121" s="3" t="s">
-        <v>134</v>
+        <v>259</v>
       </c>
       <c r="G121" s="3"/>
       <c r="H121" s="3"/>
@@ -2852,7 +3053,7 @@
       <c r="D122" s="3"/>
       <c r="E122" s="3"/>
       <c r="F122" s="3" t="s">
-        <v>22</v>
+        <v>147</v>
       </c>
       <c r="G122" s="3"/>
       <c r="H122" s="3"/>
@@ -2866,9 +3067,7 @@
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
       <c r="E123" s="3"/>
-      <c r="F123" s="3" t="s">
-        <v>150</v>
-      </c>
+      <c r="F123" s="3"/>
       <c r="G123" s="3"/>
       <c r="H123" s="3"/>
       <c r="I123" s="3"/>
@@ -2876,13 +3075,15 @@
       <c r="K123" s="3"/>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A124" s="3"/>
+      <c r="A124" s="3" t="s">
+        <v>95</v>
+      </c>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
       <c r="D124" s="3"/>
       <c r="E124" s="3"/>
       <c r="F124" s="3" t="s">
-        <v>151</v>
+        <v>130</v>
       </c>
       <c r="G124" s="3"/>
       <c r="H124" s="3"/>
@@ -2891,13 +3092,15 @@
       <c r="K124" s="3"/>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A125" s="3"/>
+      <c r="A125" s="3" t="s">
+        <v>74</v>
+      </c>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
       <c r="D125" s="3"/>
       <c r="E125" s="3"/>
       <c r="F125" s="3" t="s">
-        <v>152</v>
+        <v>121</v>
       </c>
       <c r="G125" s="3"/>
       <c r="H125" s="3"/>
@@ -2906,13 +3109,15 @@
       <c r="K125" s="3"/>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A126" s="3"/>
+      <c r="A126" s="3" t="s">
+        <v>21</v>
+      </c>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
       <c r="D126" s="3"/>
       <c r="E126" s="3"/>
       <c r="F126" s="3" t="s">
-        <v>158</v>
+        <v>131</v>
       </c>
       <c r="G126" s="3"/>
       <c r="H126" s="3"/>
@@ -2927,7 +3132,7 @@
       <c r="D127" s="3"/>
       <c r="E127" s="3"/>
       <c r="F127" s="3" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="G127" s="3"/>
       <c r="H127" s="3"/>
@@ -2935,240 +3140,245 @@
       <c r="J127" s="3"/>
       <c r="K127" s="3"/>
     </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A128" s="3"/>
+      <c r="B128" s="3"/>
+      <c r="C128" s="3"/>
+      <c r="D128" s="3"/>
+      <c r="E128" s="3"/>
+      <c r="F128" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G128" s="3"/>
+      <c r="H128" s="3"/>
+      <c r="I128" s="3"/>
+      <c r="J128" s="3"/>
+      <c r="K128" s="3"/>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A129" s="3"/>
+      <c r="B129" s="3"/>
+      <c r="C129" s="3"/>
+      <c r="D129" s="3"/>
+      <c r="E129" s="3"/>
+      <c r="F129" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="G129" s="3"/>
+      <c r="H129" s="3"/>
+      <c r="I129" s="3"/>
+      <c r="J129" s="3"/>
+      <c r="K129" s="3"/>
+    </row>
     <row r="130" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A130" s="4" t="s">
+      <c r="A130" s="3"/>
+      <c r="B130" s="3"/>
+      <c r="C130" s="3"/>
+      <c r="D130" s="3"/>
+      <c r="E130" s="3"/>
+      <c r="F130" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="G130" s="3"/>
+      <c r="H130" s="3"/>
+      <c r="I130" s="3"/>
+      <c r="J130" s="3"/>
+      <c r="K130" s="3"/>
+    </row>
+    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A131" s="3"/>
+      <c r="B131" s="3"/>
+      <c r="C131" s="3"/>
+      <c r="D131" s="3"/>
+      <c r="E131" s="3"/>
+      <c r="F131" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="G131" s="3"/>
+      <c r="H131" s="3"/>
+      <c r="I131" s="3"/>
+      <c r="J131" s="3"/>
+      <c r="K131" s="3"/>
+    </row>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A132" s="3"/>
+      <c r="B132" s="3"/>
+      <c r="C132" s="3"/>
+      <c r="D132" s="3"/>
+      <c r="E132" s="3"/>
+      <c r="F132" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G132" s="3"/>
+      <c r="H132" s="3"/>
+      <c r="I132" s="3"/>
+      <c r="J132" s="3"/>
+      <c r="K132" s="3"/>
+    </row>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A133" s="3"/>
+      <c r="B133" s="3"/>
+      <c r="C133" s="3"/>
+      <c r="D133" s="3"/>
+      <c r="E133" s="3"/>
+      <c r="F133" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="G133" s="3"/>
+      <c r="H133" s="3"/>
+      <c r="I133" s="3"/>
+      <c r="J133" s="3"/>
+      <c r="K133" s="3"/>
+    </row>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A134" s="3"/>
+      <c r="B134" s="3"/>
+      <c r="C134" s="3"/>
+      <c r="D134" s="3"/>
+      <c r="E134" s="3"/>
+      <c r="F134" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="G134" s="3"/>
+      <c r="H134" s="3"/>
+      <c r="I134" s="3"/>
+      <c r="J134" s="3"/>
+      <c r="K134" s="3"/>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A135" s="3"/>
+      <c r="B135" s="3"/>
+      <c r="C135" s="3"/>
+      <c r="D135" s="3"/>
+      <c r="E135" s="3"/>
+      <c r="F135" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G135" s="3"/>
+      <c r="H135" s="3"/>
+      <c r="I135" s="3"/>
+      <c r="J135" s="3"/>
+      <c r="K135" s="3"/>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A136" s="11"/>
+      <c r="B136" s="11"/>
+      <c r="C136" s="11"/>
+      <c r="D136" s="11"/>
+      <c r="E136" s="11"/>
+      <c r="F136" s="11"/>
+      <c r="G136" s="11"/>
+      <c r="H136" s="11"/>
+      <c r="I136" s="11"/>
+      <c r="J136" s="11"/>
+      <c r="K136" s="11"/>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A138" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B130" s="4"/>
-      <c r="C130" s="4"/>
-      <c r="D130" s="4"/>
-      <c r="E130" s="4"/>
-      <c r="F130" s="4" t="s">
+      <c r="B138" s="4"/>
+      <c r="C138" s="4"/>
+      <c r="D138" s="4"/>
+      <c r="E138" s="4"/>
+      <c r="F138" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="G138" s="4"/>
+      <c r="H138" s="4"/>
+      <c r="I138" s="4"/>
+      <c r="J138" s="4"/>
+      <c r="K138" s="4"/>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A139" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B139" s="4"/>
+      <c r="C139" s="4"/>
+      <c r="D139" s="4"/>
+      <c r="E139" s="4"/>
+      <c r="F139" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="G139" s="4"/>
+      <c r="H139" s="4"/>
+      <c r="I139" s="4"/>
+      <c r="J139" s="4"/>
+      <c r="K139" s="4"/>
+    </row>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A140" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B140" s="4"/>
+      <c r="C140" s="4"/>
+      <c r="D140" s="4"/>
+      <c r="E140" s="4"/>
+      <c r="F140" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="G140" s="4"/>
+      <c r="H140" s="4"/>
+      <c r="I140" s="4"/>
+      <c r="J140" s="4"/>
+      <c r="K140" s="4"/>
+    </row>
+    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A141" s="4"/>
+      <c r="B141" s="4"/>
+      <c r="C141" s="4"/>
+      <c r="D141" s="4"/>
+      <c r="E141" s="4"/>
+      <c r="F141" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G141" s="4"/>
+      <c r="H141" s="4"/>
+      <c r="I141" s="4"/>
+      <c r="J141" s="4"/>
+      <c r="K141" s="4"/>
+    </row>
+    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A142" s="4"/>
+      <c r="B142" s="4"/>
+      <c r="C142" s="4"/>
+      <c r="D142" s="4"/>
+      <c r="E142" s="4"/>
+      <c r="F142" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="G142" s="4"/>
+      <c r="H142" s="4"/>
+      <c r="I142" s="4"/>
+      <c r="J142" s="4"/>
+      <c r="K142" s="4"/>
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A143" s="4"/>
+      <c r="B143" s="4"/>
+      <c r="C143" s="4"/>
+      <c r="D143" s="4"/>
+      <c r="E143" s="4"/>
+      <c r="F143" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="G130" s="4"/>
-      <c r="H130" s="4"/>
-      <c r="I130" s="4"/>
-      <c r="J130" s="4"/>
-      <c r="K130" s="4"/>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A131" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="B131" s="4"/>
-      <c r="C131" s="4"/>
-      <c r="D131" s="4"/>
-      <c r="E131" s="4"/>
-      <c r="F131" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="G131" s="4"/>
-      <c r="H131" s="4"/>
-      <c r="I131" s="4"/>
-      <c r="J131" s="4"/>
-      <c r="K131" s="4"/>
-    </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A132" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B132" s="4"/>
-      <c r="C132" s="4"/>
-      <c r="D132" s="4"/>
-      <c r="E132" s="4"/>
-      <c r="F132" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="G132" s="4"/>
-      <c r="H132" s="4"/>
-      <c r="I132" s="4"/>
-      <c r="J132" s="4"/>
-      <c r="K132" s="4"/>
-    </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A133" s="4"/>
-      <c r="B133" s="4"/>
-      <c r="C133" s="4"/>
-      <c r="D133" s="4"/>
-      <c r="E133" s="4"/>
-      <c r="F133" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="G133" s="4"/>
-      <c r="H133" s="4"/>
-      <c r="I133" s="4"/>
-      <c r="J133" s="4"/>
-      <c r="K133" s="4"/>
-    </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A134" s="4"/>
-      <c r="B134" s="4"/>
-      <c r="C134" s="4"/>
-      <c r="D134" s="4"/>
-      <c r="E134" s="4"/>
-      <c r="F134" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="G134" s="4"/>
-      <c r="H134" s="4"/>
-      <c r="I134" s="4"/>
-      <c r="J134" s="4"/>
-      <c r="K134" s="4"/>
-    </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A135" s="4"/>
-      <c r="B135" s="4"/>
-      <c r="C135" s="4"/>
-      <c r="D135" s="4"/>
-      <c r="E135" s="4"/>
-      <c r="F135" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="G135" s="4"/>
-      <c r="H135" s="4"/>
-      <c r="I135" s="4"/>
-      <c r="J135" s="4"/>
-      <c r="K135" s="4"/>
-    </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A137" s="5" t="s">
+      <c r="G143" s="4"/>
+      <c r="H143" s="4"/>
+      <c r="I143" s="4"/>
+      <c r="J143" s="4"/>
+      <c r="K143" s="4"/>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A145" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B137" s="5"/>
-      <c r="C137" s="5"/>
-      <c r="D137" s="5"/>
-      <c r="E137" s="5"/>
-      <c r="F137" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="G137" s="5"/>
-      <c r="H137" s="5"/>
-      <c r="I137" s="5"/>
-      <c r="J137" s="5"/>
-      <c r="K137" s="5"/>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A138" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B138" s="5"/>
-      <c r="C138" s="5"/>
-      <c r="D138" s="5"/>
-      <c r="E138" s="5"/>
-      <c r="F138" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="G138" s="5"/>
-      <c r="H138" s="5"/>
-      <c r="I138" s="5"/>
-      <c r="J138" s="5"/>
-      <c r="K138" s="5"/>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A139" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B139" s="5"/>
-      <c r="C139" s="5"/>
-      <c r="D139" s="5"/>
-      <c r="E139" s="5"/>
-      <c r="F139" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="G139" s="5"/>
-      <c r="H139" s="5"/>
-      <c r="I139" s="5"/>
-      <c r="J139" s="5"/>
-      <c r="K139" s="5"/>
-    </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A140" s="5"/>
-      <c r="B140" s="5"/>
-      <c r="C140" s="5"/>
-      <c r="D140" s="5"/>
-      <c r="E140" s="5"/>
-      <c r="F140" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G140" s="5"/>
-      <c r="H140" s="5"/>
-      <c r="I140" s="5"/>
-      <c r="J140" s="5"/>
-      <c r="K140" s="5"/>
-    </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A141" s="5"/>
-      <c r="B141" s="5"/>
-      <c r="C141" s="5"/>
-      <c r="D141" s="5"/>
-      <c r="E141" s="5"/>
-      <c r="F141" s="5"/>
-      <c r="G141" s="5"/>
-      <c r="H141" s="5"/>
-      <c r="I141" s="5"/>
-      <c r="J141" s="5"/>
-      <c r="K141" s="5"/>
-    </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A142" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B142" s="5"/>
-      <c r="C142" s="5"/>
-      <c r="D142" s="5"/>
-      <c r="E142" s="5"/>
-      <c r="F142" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="G142" s="5"/>
-      <c r="H142" s="5"/>
-      <c r="I142" s="5"/>
-      <c r="J142" s="5"/>
-      <c r="K142" s="5"/>
-    </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A143" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B143" s="5"/>
-      <c r="C143" s="5"/>
-      <c r="D143" s="5"/>
-      <c r="E143" s="5"/>
-      <c r="F143" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="G143" s="5"/>
-      <c r="H143" s="5"/>
-      <c r="I143" s="5"/>
-      <c r="J143" s="5"/>
-      <c r="K143" s="5"/>
-    </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A144" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B144" s="5"/>
-      <c r="C144" s="5"/>
-      <c r="D144" s="5"/>
-      <c r="E144" s="5"/>
-      <c r="F144" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G144" s="5"/>
-      <c r="H144" s="5"/>
-      <c r="I144" s="5"/>
-      <c r="J144" s="5"/>
-      <c r="K144" s="5"/>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A145" s="5"/>
       <c r="B145" s="5"/>
       <c r="C145" s="5"/>
       <c r="D145" s="5"/>
       <c r="E145" s="5"/>
       <c r="F145" s="5" t="s">
-        <v>57</v>
+        <v>157</v>
       </c>
       <c r="G145" s="5"/>
       <c r="H145" s="5"/>
@@ -3177,12 +3387,16 @@
       <c r="K145" s="5"/>
     </row>
     <row r="146" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A146" s="5"/>
+      <c r="A146" s="5" t="s">
+        <v>38</v>
+      </c>
       <c r="B146" s="5"/>
       <c r="C146" s="5"/>
       <c r="D146" s="5"/>
       <c r="E146" s="5"/>
-      <c r="F146" s="5"/>
+      <c r="F146" s="5" t="s">
+        <v>158</v>
+      </c>
       <c r="G146" s="5"/>
       <c r="H146" s="5"/>
       <c r="I146" s="5"/>
@@ -3191,14 +3405,14 @@
     </row>
     <row r="147" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A147" s="5" t="s">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="B147" s="5"/>
       <c r="C147" s="5"/>
       <c r="D147" s="5"/>
       <c r="E147" s="5"/>
       <c r="F147" s="5" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="G147" s="5"/>
       <c r="H147" s="5"/>
@@ -3207,15 +3421,13 @@
       <c r="K147" s="5"/>
     </row>
     <row r="148" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A148" s="5" t="s">
-        <v>42</v>
-      </c>
+      <c r="A148" s="5"/>
       <c r="B148" s="5"/>
       <c r="C148" s="5"/>
       <c r="D148" s="5"/>
       <c r="E148" s="5"/>
       <c r="F148" s="5" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G148" s="5"/>
       <c r="H148" s="5"/>
@@ -3224,16 +3436,12 @@
       <c r="K148" s="5"/>
     </row>
     <row r="149" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A149" s="5" t="s">
-        <v>43</v>
-      </c>
+      <c r="A149" s="5"/>
       <c r="B149" s="5"/>
       <c r="C149" s="5"/>
       <c r="D149" s="5"/>
       <c r="E149" s="5"/>
-      <c r="F149" s="5" t="s">
-        <v>58</v>
-      </c>
+      <c r="F149" s="5"/>
       <c r="G149" s="5"/>
       <c r="H149" s="5"/>
       <c r="I149" s="5"/>
@@ -3241,13 +3449,15 @@
       <c r="K149" s="5"/>
     </row>
     <row r="150" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A150" s="5"/>
+      <c r="A150" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="B150" s="5"/>
       <c r="C150" s="5"/>
       <c r="D150" s="5"/>
       <c r="E150" s="5"/>
       <c r="F150" s="5" t="s">
-        <v>59</v>
+        <v>159</v>
       </c>
       <c r="G150" s="5"/>
       <c r="H150" s="5"/>
@@ -3256,12 +3466,16 @@
       <c r="K150" s="5"/>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A151" s="5"/>
+      <c r="A151" s="5" t="s">
+        <v>40</v>
+      </c>
       <c r="B151" s="5"/>
       <c r="C151" s="5"/>
       <c r="D151" s="5"/>
       <c r="E151" s="5"/>
-      <c r="F151" s="5"/>
+      <c r="F151" s="5" t="s">
+        <v>160</v>
+      </c>
       <c r="G151" s="5"/>
       <c r="H151" s="5"/>
       <c r="I151" s="5"/>
@@ -3270,14 +3484,14 @@
     </row>
     <row r="152" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A152" s="5" t="s">
-        <v>13</v>
+        <v>41</v>
       </c>
       <c r="B152" s="5"/>
       <c r="C152" s="5"/>
       <c r="D152" s="5"/>
       <c r="E152" s="5"/>
       <c r="F152" s="5" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="G152" s="5"/>
       <c r="H152" s="5"/>
@@ -3286,15 +3500,13 @@
       <c r="K152" s="5"/>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A153" s="5" t="s">
-        <v>44</v>
-      </c>
+      <c r="A153" s="5"/>
       <c r="B153" s="5"/>
       <c r="C153" s="5"/>
       <c r="D153" s="5"/>
       <c r="E153" s="5"/>
       <c r="F153" s="5" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="G153" s="5"/>
       <c r="H153" s="5"/>
@@ -3303,16 +3515,12 @@
       <c r="K153" s="5"/>
     </row>
     <row r="154" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A154" s="5" t="s">
-        <v>45</v>
-      </c>
+      <c r="A154" s="5"/>
       <c r="B154" s="5"/>
       <c r="C154" s="5"/>
       <c r="D154" s="5"/>
       <c r="E154" s="5"/>
-      <c r="F154" s="5" t="s">
-        <v>60</v>
-      </c>
+      <c r="F154" s="5"/>
       <c r="G154" s="5"/>
       <c r="H154" s="5"/>
       <c r="I154" s="5"/>
@@ -3320,13 +3528,15 @@
       <c r="K154" s="5"/>
     </row>
     <row r="155" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A155" s="5"/>
+      <c r="A155" s="5" t="s">
+        <v>13</v>
+      </c>
       <c r="B155" s="5"/>
       <c r="C155" s="5"/>
       <c r="D155" s="5"/>
       <c r="E155" s="5"/>
       <c r="F155" s="5" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="G155" s="5"/>
       <c r="H155" s="5"/>
@@ -3335,277 +3545,277 @@
       <c r="K155" s="5"/>
     </row>
     <row r="156" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A156" s="5"/>
+      <c r="A156" s="5" t="s">
+        <v>42</v>
+      </c>
       <c r="B156" s="5"/>
       <c r="C156" s="5"/>
       <c r="D156" s="5"/>
       <c r="E156" s="5"/>
-      <c r="F156" s="5"/>
+      <c r="F156" s="5" t="s">
+        <v>47</v>
+      </c>
       <c r="G156" s="5"/>
       <c r="H156" s="5"/>
       <c r="I156" s="5"/>
       <c r="J156" s="5"/>
       <c r="K156" s="5"/>
     </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A157" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="B157" s="5"/>
+      <c r="C157" s="5"/>
+      <c r="D157" s="5"/>
+      <c r="E157" s="5"/>
+      <c r="F157" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="G157" s="5"/>
+      <c r="H157" s="5"/>
+      <c r="I157" s="5"/>
+      <c r="J157" s="5"/>
+      <c r="K157" s="5"/>
+    </row>
+    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A158" s="5"/>
+      <c r="B158" s="5"/>
+      <c r="C158" s="5"/>
+      <c r="D158" s="5"/>
+      <c r="E158" s="5"/>
+      <c r="F158" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G158" s="5"/>
+      <c r="H158" s="5"/>
+      <c r="I158" s="5"/>
+      <c r="J158" s="5"/>
+      <c r="K158" s="5"/>
+    </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A159" s="6" t="s">
+      <c r="A159" s="5"/>
+      <c r="B159" s="5"/>
+      <c r="C159" s="5"/>
+      <c r="D159" s="5"/>
+      <c r="E159" s="5"/>
+      <c r="F159" s="5"/>
+      <c r="G159" s="5"/>
+      <c r="H159" s="5"/>
+      <c r="I159" s="5"/>
+      <c r="J159" s="5"/>
+      <c r="K159" s="5"/>
+    </row>
+    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A160" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B159" s="6"/>
-      <c r="C159" s="6"/>
-      <c r="D159" s="6"/>
-      <c r="E159" s="6"/>
-      <c r="F159" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="G159" s="6"/>
-      <c r="H159" s="6"/>
-      <c r="I159" s="6"/>
-      <c r="J159" s="6"/>
-      <c r="K159" s="6"/>
-    </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A160" s="6" t="s">
+      <c r="B160" s="5"/>
+      <c r="C160" s="5"/>
+      <c r="D160" s="5"/>
+      <c r="E160" s="5"/>
+      <c r="F160" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G160" s="5"/>
+      <c r="H160" s="5"/>
+      <c r="I160" s="5"/>
+      <c r="J160" s="5"/>
+      <c r="K160" s="5"/>
+    </row>
+    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A161" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B161" s="5"/>
+      <c r="C161" s="5"/>
+      <c r="D161" s="5"/>
+      <c r="E161" s="5"/>
+      <c r="F161" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="G161" s="5"/>
+      <c r="H161" s="5"/>
+      <c r="I161" s="5"/>
+      <c r="J161" s="5"/>
+      <c r="K161" s="5"/>
+    </row>
+    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A162" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B162" s="5"/>
+      <c r="C162" s="5"/>
+      <c r="D162" s="5"/>
+      <c r="E162" s="5"/>
+      <c r="F162" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="G162" s="5"/>
+      <c r="H162" s="5"/>
+      <c r="I162" s="5"/>
+      <c r="J162" s="5"/>
+      <c r="K162" s="5"/>
+    </row>
+    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A163" s="5"/>
+      <c r="B163" s="5"/>
+      <c r="C163" s="5"/>
+      <c r="D163" s="5"/>
+      <c r="E163" s="5"/>
+      <c r="F163" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="G163" s="5"/>
+      <c r="H163" s="5"/>
+      <c r="I163" s="5"/>
+      <c r="J163" s="5"/>
+      <c r="K163" s="5"/>
+    </row>
+    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A164" s="5"/>
+      <c r="B164" s="5"/>
+      <c r="C164" s="5"/>
+      <c r="D164" s="5"/>
+      <c r="E164" s="5"/>
+      <c r="F164" s="5"/>
+      <c r="G164" s="5"/>
+      <c r="H164" s="5"/>
+      <c r="I164" s="5"/>
+      <c r="J164" s="5"/>
+      <c r="K164" s="5"/>
+    </row>
+    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A167" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B167" s="6"/>
+      <c r="C167" s="6"/>
+      <c r="D167" s="6"/>
+      <c r="E167" s="6"/>
+      <c r="F167" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="G167" s="6"/>
+      <c r="H167" s="6"/>
+      <c r="I167" s="6"/>
+      <c r="J167" s="6"/>
+      <c r="K167" s="6"/>
+    </row>
+    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A168" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B160" s="6"/>
-      <c r="C160" s="6"/>
-      <c r="D160" s="6"/>
-      <c r="E160" s="6"/>
-      <c r="F160" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="G160" s="6"/>
-      <c r="H160" s="6"/>
-      <c r="I160" s="6"/>
-      <c r="J160" s="6"/>
-      <c r="K160" s="6"/>
-    </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A161" s="6" t="s">
+      <c r="B168" s="6"/>
+      <c r="C168" s="6"/>
+      <c r="D168" s="6"/>
+      <c r="E168" s="6"/>
+      <c r="F168" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="B161" s="6"/>
-      <c r="C161" s="6"/>
-      <c r="D161" s="6"/>
-      <c r="E161" s="6"/>
-      <c r="F161" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="G161" s="6"/>
-      <c r="H161" s="6"/>
-      <c r="I161" s="6"/>
-      <c r="J161" s="6"/>
-      <c r="K161" s="6"/>
-    </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A162" s="6"/>
-      <c r="B162" s="6"/>
-      <c r="C162" s="6"/>
-      <c r="D162" s="6"/>
-      <c r="E162" s="6"/>
-      <c r="F162" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="G162" s="6"/>
-      <c r="H162" s="6"/>
-      <c r="I162" s="6"/>
-      <c r="J162" s="6"/>
-      <c r="K162" s="6"/>
-    </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A164" s="8" t="s">
+      <c r="G168" s="6"/>
+      <c r="H168" s="6"/>
+      <c r="I168" s="6"/>
+      <c r="J168" s="6"/>
+      <c r="K168" s="6"/>
+    </row>
+    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A169" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B169" s="6"/>
+      <c r="C169" s="6"/>
+      <c r="D169" s="6"/>
+      <c r="E169" s="6"/>
+      <c r="F169" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="G169" s="6"/>
+      <c r="H169" s="6"/>
+      <c r="I169" s="6"/>
+      <c r="J169" s="6"/>
+      <c r="K169" s="6"/>
+    </row>
+    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A170" s="6"/>
+      <c r="B170" s="6"/>
+      <c r="C170" s="6"/>
+      <c r="D170" s="6"/>
+      <c r="E170" s="6"/>
+      <c r="F170" s="6" t="s">
+        <v>172</v>
+      </c>
+      <c r="G170" s="6"/>
+      <c r="H170" s="6"/>
+      <c r="I170" s="6"/>
+      <c r="J170" s="6"/>
+      <c r="K170" s="6"/>
+    </row>
+    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A172" s="8" t="s">
         <v>96</v>
       </c>
-      <c r="B164" s="8"/>
-      <c r="C164" s="8"/>
-      <c r="D164" s="8"/>
-      <c r="E164" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="F164" s="8"/>
-      <c r="G164" s="8"/>
-      <c r="H164" s="8"/>
-      <c r="I164" s="8"/>
-      <c r="J164" s="8"/>
-      <c r="K164" s="8"/>
-    </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A165" s="8" t="s">
+      <c r="B172" s="8"/>
+      <c r="C172" s="8"/>
+      <c r="D172" s="8"/>
+      <c r="E172" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="F172" s="8"/>
+      <c r="G172" s="8"/>
+      <c r="H172" s="8"/>
+      <c r="I172" s="8"/>
+      <c r="J172" s="8"/>
+      <c r="K172" s="8"/>
+    </row>
+    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A173" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="B165" s="8"/>
-      <c r="C165" s="8"/>
-      <c r="D165" s="8"/>
-      <c r="E165" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="F165" s="8"/>
-      <c r="G165" s="8"/>
-      <c r="H165" s="8"/>
-      <c r="I165" s="8"/>
-      <c r="J165" s="8"/>
-      <c r="K165" s="8"/>
-    </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A166" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="B166" s="8"/>
-      <c r="C166" s="8"/>
-      <c r="D166" s="8"/>
-      <c r="E166" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="F166" s="8"/>
-      <c r="G166" s="8"/>
-      <c r="H166" s="8"/>
-      <c r="I166" s="8"/>
-      <c r="J166" s="8"/>
-      <c r="K166" s="8"/>
-    </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A167" s="8"/>
-      <c r="B167" s="8"/>
-      <c r="C167" s="8"/>
-      <c r="D167" s="8"/>
-      <c r="E167" s="8" t="s">
-        <v>174</v>
-      </c>
-      <c r="F167" s="8"/>
-      <c r="G167" s="8"/>
-      <c r="H167" s="8"/>
-      <c r="I167" s="8"/>
-      <c r="J167" s="8"/>
-      <c r="K167" s="8"/>
-    </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A169" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B169" s="9"/>
-      <c r="C169" s="9"/>
-      <c r="D169" s="9"/>
-      <c r="E169" s="9"/>
-      <c r="F169" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="G169" s="9"/>
-      <c r="H169" s="9"/>
-      <c r="I169" s="9"/>
-      <c r="J169" s="9"/>
-      <c r="K169" s="9"/>
-    </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A170" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="B170" s="9"/>
-      <c r="C170" s="9"/>
-      <c r="D170" s="9"/>
-      <c r="E170" s="9"/>
-      <c r="F170" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="G170" s="9"/>
-      <c r="H170" s="9"/>
-      <c r="I170" s="9"/>
-      <c r="J170" s="9"/>
-      <c r="K170" s="9"/>
-    </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A171" s="9" t="s">
-        <v>119</v>
-      </c>
-      <c r="B171" s="9"/>
-      <c r="C171" s="9"/>
-      <c r="D171" s="9"/>
-      <c r="E171" s="9"/>
-      <c r="F171" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="G171" s="9"/>
-      <c r="H171" s="9"/>
-      <c r="I171" s="9"/>
-      <c r="J171" s="9"/>
-      <c r="K171" s="9"/>
-    </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A172" s="9"/>
-      <c r="B172" s="9"/>
-      <c r="C172" s="9"/>
-      <c r="D172" s="9"/>
-      <c r="E172" s="9"/>
-      <c r="F172" s="9"/>
-      <c r="G172" s="9"/>
-      <c r="H172" s="9"/>
-      <c r="I172" s="9"/>
-      <c r="J172" s="9"/>
-      <c r="K172" s="9"/>
-    </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A173" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B173" s="9"/>
-      <c r="C173" s="9"/>
-      <c r="D173" s="9"/>
-      <c r="E173" s="9"/>
-      <c r="F173" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="G173" s="9"/>
-      <c r="H173" s="9"/>
-      <c r="I173" s="9"/>
-      <c r="J173" s="9"/>
-      <c r="K173" s="9"/>
+      <c r="B173" s="8"/>
+      <c r="C173" s="8"/>
+      <c r="D173" s="8"/>
+      <c r="E173" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="F173" s="8"/>
+      <c r="G173" s="8"/>
+      <c r="H173" s="8"/>
+      <c r="I173" s="8"/>
+      <c r="J173" s="8"/>
+      <c r="K173" s="8"/>
     </row>
     <row r="174" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A174" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B174" s="9"/>
-      <c r="C174" s="9"/>
-      <c r="D174" s="9"/>
-      <c r="E174" s="9"/>
-      <c r="F174" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="G174" s="9"/>
-      <c r="H174" s="9"/>
-      <c r="I174" s="9"/>
-      <c r="J174" s="9"/>
-      <c r="K174" s="9"/>
+      <c r="A174" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="B174" s="8"/>
+      <c r="C174" s="8"/>
+      <c r="D174" s="8"/>
+      <c r="E174" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="F174" s="8"/>
+      <c r="G174" s="8"/>
+      <c r="H174" s="8"/>
+      <c r="I174" s="8"/>
+      <c r="J174" s="8"/>
+      <c r="K174" s="8"/>
     </row>
     <row r="175" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A175" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B175" s="9"/>
-      <c r="C175" s="9"/>
-      <c r="D175" s="9"/>
-      <c r="E175" s="9"/>
-      <c r="F175" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="G175" s="9"/>
-      <c r="H175" s="9"/>
-      <c r="I175" s="9"/>
-      <c r="J175" s="9"/>
-      <c r="K175" s="9"/>
-    </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A176" s="9"/>
-      <c r="B176" s="9"/>
-      <c r="C176" s="9"/>
-      <c r="D176" s="9"/>
-      <c r="E176" s="9"/>
-      <c r="F176" s="9"/>
-      <c r="G176" s="9"/>
-      <c r="H176" s="9"/>
-      <c r="I176" s="9"/>
-      <c r="J176" s="9"/>
-      <c r="K176" s="9"/>
+      <c r="A175" s="8"/>
+      <c r="B175" s="8"/>
+      <c r="C175" s="8"/>
+      <c r="D175" s="8"/>
+      <c r="E175" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="F175" s="8"/>
+      <c r="G175" s="8"/>
+      <c r="H175" s="8"/>
+      <c r="I175" s="8"/>
+      <c r="J175" s="8"/>
+      <c r="K175" s="8"/>
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A177" s="9" t="s">
@@ -3616,7 +3826,7 @@
       <c r="D177" s="9"/>
       <c r="E177" s="9"/>
       <c r="F177" s="9" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="G177" s="9"/>
       <c r="H177" s="9"/>
@@ -3626,14 +3836,14 @@
     </row>
     <row r="178" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A178" s="9" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B178" s="9"/>
       <c r="C178" s="9"/>
       <c r="D178" s="9"/>
       <c r="E178" s="9"/>
       <c r="F178" s="9" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G178" s="9"/>
       <c r="H178" s="9"/>
@@ -3643,14 +3853,14 @@
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A179" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B179" s="9"/>
       <c r="C179" s="9"/>
       <c r="D179" s="9"/>
       <c r="E179" s="9"/>
       <c r="F179" s="9" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G179" s="9"/>
       <c r="H179" s="9"/>
@@ -3680,7 +3890,7 @@
       <c r="D181" s="9"/>
       <c r="E181" s="9"/>
       <c r="F181" s="9" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="G181" s="9"/>
       <c r="H181" s="9"/>
@@ -3690,14 +3900,14 @@
     </row>
     <row r="182" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A182" s="9" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B182" s="9"/>
       <c r="C182" s="9"/>
       <c r="D182" s="9"/>
       <c r="E182" s="9"/>
       <c r="F182" s="9" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="G182" s="9"/>
       <c r="H182" s="9"/>
@@ -3707,14 +3917,14 @@
     </row>
     <row r="183" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A183" s="9" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="B183" s="9"/>
       <c r="C183" s="9"/>
       <c r="D183" s="9"/>
       <c r="E183" s="9"/>
       <c r="F183" s="9" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G183" s="9"/>
       <c r="H183" s="9"/>
@@ -3722,6 +3932,977 @@
       <c r="J183" s="9"/>
       <c r="K183" s="9"/>
     </row>
+    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A184" s="9"/>
+      <c r="B184" s="9"/>
+      <c r="C184" s="9"/>
+      <c r="D184" s="9"/>
+      <c r="E184" s="9"/>
+      <c r="F184" s="9"/>
+      <c r="G184" s="9"/>
+      <c r="H184" s="9"/>
+      <c r="I184" s="9"/>
+      <c r="J184" s="9"/>
+      <c r="K184" s="9"/>
+    </row>
+    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A185" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B185" s="9"/>
+      <c r="C185" s="9"/>
+      <c r="D185" s="9"/>
+      <c r="E185" s="9"/>
+      <c r="F185" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="G185" s="9"/>
+      <c r="H185" s="9"/>
+      <c r="I185" s="9"/>
+      <c r="J185" s="9"/>
+      <c r="K185" s="9"/>
+    </row>
+    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A186" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="B186" s="9"/>
+      <c r="C186" s="9"/>
+      <c r="D186" s="9"/>
+      <c r="E186" s="9"/>
+      <c r="F186" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="G186" s="9"/>
+      <c r="H186" s="9"/>
+      <c r="I186" s="9"/>
+      <c r="J186" s="9"/>
+      <c r="K186" s="9"/>
+    </row>
+    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A187" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="B187" s="9"/>
+      <c r="C187" s="9"/>
+      <c r="D187" s="9"/>
+      <c r="E187" s="9"/>
+      <c r="F187" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="G187" s="9"/>
+      <c r="H187" s="9"/>
+      <c r="I187" s="9"/>
+      <c r="J187" s="9"/>
+      <c r="K187" s="9"/>
+    </row>
+    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A188" s="9"/>
+      <c r="B188" s="9"/>
+      <c r="C188" s="9"/>
+      <c r="D188" s="9"/>
+      <c r="E188" s="9"/>
+      <c r="F188" s="9"/>
+      <c r="G188" s="9"/>
+      <c r="H188" s="9"/>
+      <c r="I188" s="9"/>
+      <c r="J188" s="9"/>
+      <c r="K188" s="9"/>
+    </row>
+    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A189" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B189" s="9"/>
+      <c r="C189" s="9"/>
+      <c r="D189" s="9"/>
+      <c r="E189" s="9"/>
+      <c r="F189" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="G189" s="9"/>
+      <c r="H189" s="9"/>
+      <c r="I189" s="9"/>
+      <c r="J189" s="9"/>
+      <c r="K189" s="9"/>
+    </row>
+    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A190" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="B190" s="9"/>
+      <c r="C190" s="9"/>
+      <c r="D190" s="9"/>
+      <c r="E190" s="9"/>
+      <c r="F190" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="G190" s="9"/>
+      <c r="H190" s="9"/>
+      <c r="I190" s="9"/>
+      <c r="J190" s="9"/>
+      <c r="K190" s="9"/>
+    </row>
+    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A191" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="B191" s="9"/>
+      <c r="C191" s="9"/>
+      <c r="D191" s="9"/>
+      <c r="E191" s="9"/>
+      <c r="F191" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G191" s="9"/>
+      <c r="H191" s="9"/>
+      <c r="I191" s="9"/>
+      <c r="J191" s="9"/>
+      <c r="K191" s="9"/>
+    </row>
+    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A193" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B193" s="4"/>
+      <c r="C193" s="4"/>
+      <c r="D193" s="4"/>
+      <c r="E193" s="4"/>
+      <c r="F193" s="4" t="s">
+        <v>250</v>
+      </c>
+      <c r="G193" s="4"/>
+      <c r="H193" s="4"/>
+      <c r="I193" s="4"/>
+      <c r="J193" s="4"/>
+      <c r="K193" s="4"/>
+    </row>
+    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A194" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B194" s="4"/>
+      <c r="C194" s="4"/>
+      <c r="D194" s="4"/>
+      <c r="E194" s="4"/>
+      <c r="F194" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="G194" s="4"/>
+      <c r="H194" s="4"/>
+      <c r="I194" s="4"/>
+      <c r="J194" s="4"/>
+      <c r="K194" s="4"/>
+    </row>
+    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A195" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B195" s="4"/>
+      <c r="C195" s="4"/>
+      <c r="D195" s="4"/>
+      <c r="E195" s="4"/>
+      <c r="F195" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="G195" s="4"/>
+      <c r="H195" s="4"/>
+      <c r="I195" s="4"/>
+      <c r="J195" s="4"/>
+      <c r="K195" s="4"/>
+    </row>
+    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A196" s="4"/>
+      <c r="B196" s="4"/>
+      <c r="C196" s="4"/>
+      <c r="D196" s="4"/>
+      <c r="E196" s="4"/>
+      <c r="F196" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="G196" s="4"/>
+      <c r="H196" s="4"/>
+      <c r="I196" s="4"/>
+      <c r="J196" s="4"/>
+      <c r="K196" s="4"/>
+    </row>
+    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A197" s="4"/>
+      <c r="B197" s="4"/>
+      <c r="C197" s="4"/>
+      <c r="D197" s="4"/>
+      <c r="E197" s="4"/>
+      <c r="F197" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="G197" s="4"/>
+      <c r="H197" s="4"/>
+      <c r="I197" s="4"/>
+      <c r="J197" s="4"/>
+      <c r="K197" s="4"/>
+    </row>
+    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A198" s="4"/>
+      <c r="B198" s="4"/>
+      <c r="C198" s="4"/>
+      <c r="D198" s="4"/>
+      <c r="E198" s="4"/>
+      <c r="F198" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="G198" s="4"/>
+      <c r="H198" s="4"/>
+      <c r="I198" s="4"/>
+      <c r="J198" s="4"/>
+      <c r="K198" s="4"/>
+    </row>
+    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A199" s="4"/>
+      <c r="B199" s="4"/>
+      <c r="C199" s="4"/>
+      <c r="D199" s="4"/>
+      <c r="E199" s="4"/>
+      <c r="F199" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="G199" s="4"/>
+      <c r="H199" s="4"/>
+      <c r="I199" s="4"/>
+      <c r="J199" s="4"/>
+      <c r="K199" s="4"/>
+    </row>
+    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A200" s="4"/>
+      <c r="B200" s="4"/>
+      <c r="C200" s="4"/>
+      <c r="D200" s="4"/>
+      <c r="E200" s="4"/>
+      <c r="F200" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="G200" s="4"/>
+      <c r="H200" s="4"/>
+      <c r="I200" s="4"/>
+      <c r="J200" s="4"/>
+      <c r="K200" s="4"/>
+    </row>
+    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A201" s="4"/>
+      <c r="B201" s="4"/>
+      <c r="C201" s="4"/>
+      <c r="D201" s="4"/>
+      <c r="E201" s="4"/>
+      <c r="F201" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="G201" s="4"/>
+      <c r="H201" s="4"/>
+      <c r="I201" s="4"/>
+      <c r="J201" s="4"/>
+      <c r="K201" s="4"/>
+    </row>
+    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A202" s="4"/>
+      <c r="B202" s="4"/>
+      <c r="C202" s="4"/>
+      <c r="D202" s="4"/>
+      <c r="E202" s="4"/>
+      <c r="F202" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="G202" s="4"/>
+      <c r="H202" s="4"/>
+      <c r="I202" s="4"/>
+      <c r="J202" s="4"/>
+      <c r="K202" s="4"/>
+    </row>
+    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A203" s="4"/>
+      <c r="B203" s="4"/>
+      <c r="C203" s="4"/>
+      <c r="D203" s="4"/>
+      <c r="E203" s="4"/>
+      <c r="F203" s="4" t="s">
+        <v>200</v>
+      </c>
+      <c r="G203" s="4"/>
+      <c r="H203" s="4"/>
+      <c r="I203" s="4"/>
+      <c r="J203" s="4"/>
+      <c r="K203" s="4"/>
+    </row>
+    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A204" s="4"/>
+      <c r="B204" s="4"/>
+      <c r="C204" s="4"/>
+      <c r="D204" s="4"/>
+      <c r="E204" s="4"/>
+      <c r="F204" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="G204" s="4"/>
+      <c r="H204" s="4"/>
+      <c r="I204" s="4"/>
+      <c r="J204" s="4"/>
+      <c r="K204" s="4"/>
+    </row>
+    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A205" s="4"/>
+      <c r="B205" s="4"/>
+      <c r="C205" s="4"/>
+      <c r="D205" s="4"/>
+      <c r="E205" s="4"/>
+      <c r="F205" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="G205" s="4"/>
+      <c r="H205" s="4"/>
+      <c r="I205" s="4"/>
+      <c r="J205" s="4"/>
+      <c r="K205" s="4"/>
+    </row>
+    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A206" s="4"/>
+      <c r="B206" s="4"/>
+      <c r="C206" s="4"/>
+      <c r="D206" s="4"/>
+      <c r="E206" s="4"/>
+      <c r="F206" s="4"/>
+      <c r="G206" s="4"/>
+      <c r="H206" s="4"/>
+      <c r="I206" s="4"/>
+      <c r="J206" s="4"/>
+      <c r="K206" s="4"/>
+    </row>
+    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A207" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B207" s="4"/>
+      <c r="C207" s="4"/>
+      <c r="D207" s="4"/>
+      <c r="E207" s="4"/>
+      <c r="F207" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="G207" s="4"/>
+      <c r="H207" s="4"/>
+      <c r="I207" s="4"/>
+      <c r="J207" s="4"/>
+      <c r="K207" s="4"/>
+    </row>
+    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A208" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B208" s="4"/>
+      <c r="C208" s="4"/>
+      <c r="D208" s="4"/>
+      <c r="E208" s="4"/>
+      <c r="F208" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="G208" s="4"/>
+      <c r="H208" s="4"/>
+      <c r="I208" s="4"/>
+      <c r="J208" s="4"/>
+      <c r="K208" s="4"/>
+    </row>
+    <row r="209" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A209" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B209" s="4"/>
+      <c r="C209" s="4"/>
+      <c r="D209" s="4"/>
+      <c r="E209" s="4"/>
+      <c r="F209" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="G209" s="4"/>
+      <c r="H209" s="4"/>
+      <c r="I209" s="4"/>
+      <c r="J209" s="4"/>
+      <c r="K209" s="4"/>
+    </row>
+    <row r="210" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A210" s="4"/>
+      <c r="B210" s="4"/>
+      <c r="C210" s="4"/>
+      <c r="D210" s="4"/>
+      <c r="E210" s="4"/>
+      <c r="F210" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="G210" s="4"/>
+      <c r="H210" s="4"/>
+      <c r="I210" s="4"/>
+      <c r="J210" s="4"/>
+      <c r="K210" s="4"/>
+    </row>
+    <row r="211" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A211" s="4"/>
+      <c r="B211" s="4"/>
+      <c r="C211" s="4"/>
+      <c r="D211" s="4"/>
+      <c r="E211" s="4"/>
+      <c r="F211" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="G211" s="4"/>
+      <c r="H211" s="4"/>
+      <c r="I211" s="4"/>
+      <c r="J211" s="4"/>
+      <c r="K211" s="4"/>
+    </row>
+    <row r="212" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A212" s="4"/>
+      <c r="B212" s="4"/>
+      <c r="C212" s="4"/>
+      <c r="D212" s="4"/>
+      <c r="E212" s="4"/>
+      <c r="F212" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="G212" s="4"/>
+      <c r="H212" s="4"/>
+      <c r="I212" s="4"/>
+      <c r="J212" s="4"/>
+      <c r="K212" s="4"/>
+    </row>
+    <row r="213" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A213" s="4"/>
+      <c r="B213" s="4"/>
+      <c r="C213" s="4"/>
+      <c r="D213" s="4"/>
+      <c r="E213" s="4"/>
+      <c r="F213" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="G213" s="4"/>
+      <c r="H213" s="4"/>
+      <c r="I213" s="4"/>
+      <c r="J213" s="4"/>
+      <c r="K213" s="4"/>
+    </row>
+    <row r="214" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A214" s="4"/>
+      <c r="B214" s="4"/>
+      <c r="C214" s="4"/>
+      <c r="D214" s="4"/>
+      <c r="E214" s="4"/>
+      <c r="F214" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="G214" s="4"/>
+      <c r="H214" s="4"/>
+      <c r="I214" s="4"/>
+      <c r="J214" s="4"/>
+      <c r="K214" s="4"/>
+    </row>
+    <row r="215" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A215" s="4"/>
+      <c r="B215" s="4"/>
+      <c r="C215" s="4"/>
+      <c r="D215" s="4"/>
+      <c r="E215" s="4"/>
+      <c r="F215" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="G215" s="4"/>
+      <c r="H215" s="4"/>
+      <c r="I215" s="4"/>
+      <c r="J215" s="4"/>
+      <c r="K215" s="4"/>
+    </row>
+    <row r="216" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A216" s="4"/>
+      <c r="B216" s="4"/>
+      <c r="C216" s="4"/>
+      <c r="D216" s="4"/>
+      <c r="E216" s="4"/>
+      <c r="F216" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="G216" s="4"/>
+      <c r="H216" s="4"/>
+      <c r="I216" s="4"/>
+      <c r="J216" s="4"/>
+      <c r="K216" s="4"/>
+    </row>
+    <row r="217" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A217" s="4"/>
+      <c r="B217" s="4"/>
+      <c r="C217" s="4"/>
+      <c r="D217" s="4"/>
+      <c r="E217" s="4"/>
+      <c r="F217" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="G217" s="4"/>
+      <c r="H217" s="4"/>
+      <c r="I217" s="4"/>
+      <c r="J217" s="4"/>
+      <c r="K217" s="4"/>
+    </row>
+    <row r="218" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A218" s="4"/>
+      <c r="B218" s="4"/>
+      <c r="C218" s="4"/>
+      <c r="D218" s="4"/>
+      <c r="E218" s="4"/>
+      <c r="F218" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="G218" s="4"/>
+      <c r="H218" s="4"/>
+      <c r="I218" s="4"/>
+      <c r="J218" s="4"/>
+      <c r="K218" s="4"/>
+    </row>
+    <row r="219" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A219" s="4"/>
+      <c r="B219" s="4"/>
+      <c r="C219" s="4"/>
+      <c r="D219" s="4"/>
+      <c r="E219" s="4"/>
+      <c r="F219" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="G219" s="4"/>
+      <c r="H219" s="4"/>
+      <c r="I219" s="4"/>
+      <c r="J219" s="4"/>
+      <c r="K219" s="4"/>
+    </row>
+    <row r="220" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A220" s="4"/>
+      <c r="B220" s="4"/>
+      <c r="C220" s="4"/>
+      <c r="D220" s="4"/>
+      <c r="E220" s="4"/>
+      <c r="F220" s="4"/>
+      <c r="G220" s="4"/>
+      <c r="H220" s="4"/>
+      <c r="I220" s="4"/>
+      <c r="J220" s="4"/>
+      <c r="K220" s="4"/>
+    </row>
+    <row r="221" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A221" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B221" s="4"/>
+      <c r="C221" s="4"/>
+      <c r="D221" s="4"/>
+      <c r="E221" s="4"/>
+      <c r="F221" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="G221" s="4"/>
+      <c r="H221" s="4"/>
+      <c r="I221" s="4"/>
+      <c r="J221" s="4"/>
+      <c r="K221" s="4"/>
+    </row>
+    <row r="222" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A222" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B222" s="4"/>
+      <c r="C222" s="4"/>
+      <c r="D222" s="4"/>
+      <c r="E222" s="4"/>
+      <c r="F222" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="G222" s="4"/>
+      <c r="H222" s="4"/>
+      <c r="I222" s="4"/>
+      <c r="J222" s="4"/>
+      <c r="K222" s="4"/>
+    </row>
+    <row r="223" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A223" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="B223" s="4"/>
+      <c r="C223" s="4"/>
+      <c r="D223" s="4"/>
+      <c r="E223" s="4"/>
+      <c r="F223" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="G223" s="4"/>
+      <c r="H223" s="4"/>
+      <c r="I223" s="4"/>
+      <c r="J223" s="4"/>
+      <c r="K223" s="4"/>
+    </row>
+    <row r="224" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A224" s="4"/>
+      <c r="B224" s="4"/>
+      <c r="C224" s="4"/>
+      <c r="D224" s="4"/>
+      <c r="E224" s="4"/>
+      <c r="F224" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="G224" s="4"/>
+      <c r="H224" s="4"/>
+      <c r="I224" s="4"/>
+      <c r="J224" s="4"/>
+      <c r="K224" s="4"/>
+    </row>
+    <row r="225" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A225" s="4"/>
+      <c r="B225" s="4"/>
+      <c r="C225" s="4"/>
+      <c r="D225" s="4"/>
+      <c r="E225" s="4"/>
+      <c r="F225" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="G225" s="4"/>
+      <c r="H225" s="4"/>
+      <c r="I225" s="4"/>
+      <c r="J225" s="4"/>
+      <c r="K225" s="4"/>
+    </row>
+    <row r="226" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A226" s="4"/>
+      <c r="B226" s="4"/>
+      <c r="C226" s="4"/>
+      <c r="D226" s="4"/>
+      <c r="E226" s="4"/>
+      <c r="F226" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="G226" s="4"/>
+      <c r="H226" s="4"/>
+      <c r="I226" s="4"/>
+      <c r="J226" s="4"/>
+      <c r="K226" s="4"/>
+    </row>
+    <row r="227" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A227" s="4"/>
+      <c r="B227" s="4"/>
+      <c r="C227" s="4"/>
+      <c r="D227" s="4"/>
+      <c r="E227" s="4"/>
+      <c r="F227" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="G227" s="4"/>
+      <c r="H227" s="4"/>
+      <c r="I227" s="4"/>
+      <c r="J227" s="4"/>
+      <c r="K227" s="4"/>
+    </row>
+    <row r="228" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A228" s="4"/>
+      <c r="B228" s="4"/>
+      <c r="C228" s="4"/>
+      <c r="D228" s="4"/>
+      <c r="E228" s="4"/>
+      <c r="F228" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="G228" s="4"/>
+      <c r="H228" s="4"/>
+      <c r="I228" s="4"/>
+      <c r="J228" s="4"/>
+      <c r="K228" s="4"/>
+    </row>
+    <row r="229" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A229" s="4"/>
+      <c r="B229" s="4"/>
+      <c r="C229" s="4"/>
+      <c r="D229" s="4"/>
+      <c r="E229" s="4"/>
+      <c r="F229" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="G229" s="4"/>
+      <c r="H229" s="4"/>
+      <c r="I229" s="4"/>
+      <c r="J229" s="4"/>
+      <c r="K229" s="4"/>
+    </row>
+    <row r="230" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A230" s="4"/>
+      <c r="B230" s="4"/>
+      <c r="C230" s="4"/>
+      <c r="D230" s="4"/>
+      <c r="E230" s="4"/>
+      <c r="F230" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="G230" s="4"/>
+      <c r="H230" s="4"/>
+      <c r="I230" s="4"/>
+      <c r="J230" s="4"/>
+      <c r="K230" s="4"/>
+    </row>
+    <row r="231" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A231" s="4"/>
+      <c r="B231" s="4"/>
+      <c r="C231" s="4"/>
+      <c r="D231" s="4"/>
+      <c r="E231" s="4"/>
+      <c r="F231" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="G231" s="4"/>
+      <c r="H231" s="4"/>
+      <c r="I231" s="4"/>
+      <c r="J231" s="4"/>
+      <c r="K231" s="4"/>
+    </row>
+    <row r="232" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A232" s="4"/>
+      <c r="B232" s="4"/>
+      <c r="C232" s="4"/>
+      <c r="D232" s="4"/>
+      <c r="E232" s="4"/>
+      <c r="F232" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="G232" s="4"/>
+      <c r="H232" s="4"/>
+      <c r="I232" s="4"/>
+      <c r="J232" s="4"/>
+      <c r="K232" s="4"/>
+    </row>
+    <row r="233" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A233" s="4"/>
+      <c r="B233" s="4"/>
+      <c r="C233" s="4"/>
+      <c r="D233" s="4"/>
+      <c r="E233" s="4"/>
+      <c r="F233" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="G233" s="4"/>
+      <c r="H233" s="4"/>
+      <c r="I233" s="4"/>
+      <c r="J233" s="4"/>
+      <c r="K233" s="4"/>
+    </row>
+    <row r="234" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A234" s="4"/>
+      <c r="B234" s="4"/>
+      <c r="C234" s="4"/>
+      <c r="D234" s="4"/>
+      <c r="E234" s="4"/>
+      <c r="F234" s="4"/>
+      <c r="G234" s="4"/>
+      <c r="H234" s="4"/>
+      <c r="I234" s="4"/>
+      <c r="J234" s="4"/>
+      <c r="K234" s="4"/>
+    </row>
+    <row r="235" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A235" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B235" s="4"/>
+      <c r="C235" s="4"/>
+      <c r="D235" s="4"/>
+      <c r="E235" s="4"/>
+      <c r="F235" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="G235" s="4"/>
+      <c r="H235" s="4"/>
+      <c r="I235" s="4"/>
+      <c r="J235" s="4"/>
+      <c r="K235" s="4"/>
+    </row>
+    <row r="236" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A236" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B236" s="4"/>
+      <c r="C236" s="4"/>
+      <c r="D236" s="4"/>
+      <c r="E236" s="4"/>
+      <c r="F236" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="G236" s="4"/>
+      <c r="H236" s="4"/>
+      <c r="I236" s="4"/>
+      <c r="J236" s="4"/>
+      <c r="K236" s="4"/>
+    </row>
+    <row r="237" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A237" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B237" s="4"/>
+      <c r="C237" s="4"/>
+      <c r="D237" s="4"/>
+      <c r="E237" s="4"/>
+      <c r="F237" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="G237" s="4"/>
+      <c r="H237" s="4"/>
+      <c r="I237" s="4"/>
+      <c r="J237" s="4"/>
+      <c r="K237" s="4"/>
+    </row>
+    <row r="238" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A238" s="4"/>
+      <c r="B238" s="4"/>
+      <c r="C238" s="4"/>
+      <c r="D238" s="4"/>
+      <c r="E238" s="4"/>
+      <c r="F238" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="G238" s="4"/>
+      <c r="H238" s="4"/>
+      <c r="I238" s="4"/>
+      <c r="J238" s="4"/>
+      <c r="K238" s="4"/>
+    </row>
+    <row r="239" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A239" s="4"/>
+      <c r="B239" s="4"/>
+      <c r="C239" s="4"/>
+      <c r="D239" s="4"/>
+      <c r="E239" s="4"/>
+      <c r="F239" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="G239" s="4"/>
+      <c r="H239" s="4"/>
+      <c r="I239" s="4"/>
+      <c r="J239" s="4"/>
+      <c r="K239" s="4"/>
+    </row>
+    <row r="240" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A240" s="4"/>
+      <c r="B240" s="4"/>
+      <c r="C240" s="4"/>
+      <c r="D240" s="4"/>
+      <c r="E240" s="4"/>
+      <c r="F240" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="G240" s="4"/>
+      <c r="H240" s="4"/>
+      <c r="I240" s="4"/>
+      <c r="J240" s="4"/>
+      <c r="K240" s="4"/>
+    </row>
+    <row r="241" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A241" s="4"/>
+      <c r="B241" s="4"/>
+      <c r="C241" s="4"/>
+      <c r="D241" s="4"/>
+      <c r="E241" s="4"/>
+      <c r="F241" s="4" t="s">
+        <v>230</v>
+      </c>
+      <c r="G241" s="4"/>
+      <c r="H241" s="4"/>
+      <c r="I241" s="4"/>
+      <c r="J241" s="4"/>
+      <c r="K241" s="4"/>
+    </row>
+    <row r="242" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A242" s="4"/>
+      <c r="B242" s="4"/>
+      <c r="C242" s="4"/>
+      <c r="D242" s="4"/>
+      <c r="E242" s="4"/>
+      <c r="F242" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="G242" s="4"/>
+      <c r="H242" s="4"/>
+      <c r="I242" s="4"/>
+      <c r="J242" s="4"/>
+      <c r="K242" s="4"/>
+    </row>
+    <row r="243" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A243" s="4"/>
+      <c r="B243" s="4"/>
+      <c r="C243" s="4"/>
+      <c r="D243" s="4"/>
+      <c r="E243" s="4"/>
+      <c r="F243" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="G243" s="4"/>
+      <c r="H243" s="4"/>
+      <c r="I243" s="4"/>
+      <c r="J243" s="4"/>
+      <c r="K243" s="4"/>
+    </row>
+    <row r="244" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A244" s="4"/>
+      <c r="B244" s="4"/>
+      <c r="C244" s="4"/>
+      <c r="D244" s="4"/>
+      <c r="E244" s="4"/>
+      <c r="F244" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="G244" s="4"/>
+      <c r="H244" s="4"/>
+      <c r="I244" s="4"/>
+      <c r="J244" s="4"/>
+      <c r="K244" s="4"/>
+    </row>
+    <row r="245" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A245" s="4"/>
+      <c r="B245" s="4"/>
+      <c r="C245" s="4"/>
+      <c r="D245" s="4"/>
+      <c r="E245" s="4"/>
+      <c r="F245" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="G245" s="4"/>
+      <c r="H245" s="4"/>
+      <c r="I245" s="4"/>
+      <c r="J245" s="4"/>
+      <c r="K245" s="4"/>
+    </row>
+    <row r="246" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A246" s="4"/>
+      <c r="B246" s="4"/>
+      <c r="C246" s="4"/>
+      <c r="D246" s="4"/>
+      <c r="E246" s="4"/>
+      <c r="F246" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="G246" s="4"/>
+      <c r="H246" s="4"/>
+      <c r="I246" s="4"/>
+      <c r="J246" s="4"/>
+      <c r="K246" s="4"/>
+    </row>
+    <row r="247" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A247" s="4"/>
+      <c r="B247" s="4"/>
+      <c r="C247" s="4"/>
+      <c r="D247" s="4"/>
+      <c r="E247" s="4"/>
+      <c r="F247" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="G247" s="4"/>
+      <c r="H247" s="4"/>
+      <c r="I247" s="4"/>
+      <c r="J247" s="4"/>
+      <c r="K247" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Platform type updated in user stories and database
</commit_message>
<xml_diff>
--- a/DBMS Game Store Docs/User Stories.xlsx
+++ b/DBMS Game Store Docs/User Stories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryanc\Desktop\final_year_project\DBMS Game Store Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1997A2F9-BB7A-48F5-91BF-D015654D870B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518A0D7B-13FE-4149-B0D8-078C870DFE1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{91133E6D-6CC4-4AFD-BF36-5C9837FF4593}"/>
+    <workbookView xWindow="60" yWindow="0" windowWidth="13410" windowHeight="16305" xr2:uid="{91133E6D-6CC4-4AFD-BF36-5C9837FF4593}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="253">
   <si>
     <t>As a admin,</t>
   </si>
@@ -152,9 +152,6 @@
     <t xml:space="preserve">so I can ensure delivery. </t>
   </si>
   <si>
-    <t>I want to create publications for stock,</t>
-  </si>
-  <si>
     <t>so I can sell them.</t>
   </si>
   <si>
@@ -167,36 +164,12 @@
     <t>I want to update stock,</t>
   </si>
   <si>
-    <t>so I can sell new publications.</t>
-  </si>
-  <si>
     <t>I want to delete stock</t>
   </si>
   <si>
-    <t>so I can not sell old publications.</t>
-  </si>
-  <si>
-    <t>Verify new PS4 games are updated to stock.</t>
-  </si>
-  <si>
-    <t>Verify new Xbox games are updated to stock.</t>
-  </si>
-  <si>
-    <t>Verify old PS4 games are deleted from the stock.</t>
-  </si>
-  <si>
-    <t>Verify old Xbox games are deleted from the stock.</t>
-  </si>
-  <si>
     <t>I want to have payments computed automatically,</t>
   </si>
   <si>
-    <t>Verify system creates PS4 game stock quantity details 0&gt; &amp; &lt;1000.</t>
-  </si>
-  <si>
-    <t>Verify system creates Xbox game stock quantity details 0&gt; &amp; &lt;1000.</t>
-  </si>
-  <si>
     <t>Verify employee's name is created 0&gt; &amp; &lt;10.</t>
   </si>
   <si>
@@ -206,24 +179,6 @@
     <t>Verify employee's phone number is created 0&gt; &amp; &lt;10.</t>
   </si>
   <si>
-    <t>Verify system reads PS4 game stock quantity details.</t>
-  </si>
-  <si>
-    <t>Verify system reads Xbox game stock quantity details.</t>
-  </si>
-  <si>
-    <t>Verify system updates PS4 game stock quantity details.</t>
-  </si>
-  <si>
-    <t>Verify system updates Xbox game stock quantity details.</t>
-  </si>
-  <si>
-    <t>Verify system deletes PS4 games stock quantity details.</t>
-  </si>
-  <si>
-    <t>Verify system deletes Xbox games stock quantity details.</t>
-  </si>
-  <si>
     <t>Verify manager's name is created 0&gt; &amp; &lt;10.</t>
   </si>
   <si>
@@ -335,27 +290,9 @@
     <t>so I can calculate sales.</t>
   </si>
   <si>
-    <t>Verify a ps4 games sold cost is displayed to the manager.</t>
-  </si>
-  <si>
-    <t>Verify a xbox games sold cost is displayed to the manager.</t>
-  </si>
-  <si>
     <t>I want to create a list of my favourite games,</t>
   </si>
   <si>
-    <t>Verify wishlist for a PS4 game title is created.</t>
-  </si>
-  <si>
-    <t>Verify wishlist for a PS4 game title is read.</t>
-  </si>
-  <si>
-    <t>Verify wishlist for a PS4 game title is updated.</t>
-  </si>
-  <si>
-    <t>Verify wishlist for a PS4 game title is deleted.</t>
-  </si>
-  <si>
     <t>I want to read a list of my favourite games,</t>
   </si>
   <si>
@@ -377,18 +314,6 @@
     <t>so I can view the games I've bought.</t>
   </si>
   <si>
-    <t>Verify wishlist for a Xbox game title is created.</t>
-  </si>
-  <si>
-    <t>Verify wishlist for a Xbox game title is read.</t>
-  </si>
-  <si>
-    <t>Verify wishlist for a Xbox game title is updated.</t>
-  </si>
-  <si>
-    <t>Verify wishlist for a Xbox game title is deleted.</t>
-  </si>
-  <si>
     <t>so I can not have to search them later.</t>
   </si>
   <si>
@@ -509,18 +434,6 @@
     <t>Verify game price is deleted.</t>
   </si>
   <si>
-    <t>Verify PS4 game title is created.</t>
-  </si>
-  <si>
-    <t>Verify Xbox game title is created.</t>
-  </si>
-  <si>
-    <t>Verify PS4 game title is read.</t>
-  </si>
-  <si>
-    <t>Verify Xbox game title is read.</t>
-  </si>
-  <si>
     <t>Verify wishlist is created.</t>
   </si>
   <si>
@@ -536,24 +449,12 @@
     <t>Verify system prints platform.</t>
   </si>
   <si>
-    <t>Verify system prints customer game title.</t>
-  </si>
-  <si>
     <t>Verify system prints customer summary.</t>
   </si>
   <si>
     <t>I want to know customer history,</t>
   </si>
   <si>
-    <t>Verify system prints game number.</t>
-  </si>
-  <si>
-    <t>Verify system prints manager number.</t>
-  </si>
-  <si>
-    <t>Verify manager number is displayed.</t>
-  </si>
-  <si>
     <t>Verify order number is displayed.</t>
   </si>
   <si>
@@ -620,33 +521,6 @@
     <t>so I can let customers buy games and music.</t>
   </si>
   <si>
-    <t>Verfiy payment amount is created for music.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is created for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is created for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is created for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is created for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is created for music.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is created for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is created for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is created for music.</t>
-  </si>
-  <si>
     <t>I want to read paymets,</t>
   </si>
   <si>
@@ -659,96 +533,6 @@
     <t>I want to create payments,</t>
   </si>
   <si>
-    <t>Verify order id is read for payments.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is read for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is read for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is read for music.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is read for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is read for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is read for music.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is read for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is read for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is read for music.</t>
-  </si>
-  <si>
-    <t>Verify order id is updated for payments.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is updated for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is updated for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is updated for music.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is updated for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is updated for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is updated for music.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is updated for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is updated for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is updated for music.</t>
-  </si>
-  <si>
-    <t>Verify order id is deleted for payments.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is deleted for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is deleted for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment amount is deleted for music.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is deleted for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is deleted for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment status is deleted for music.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is deleted for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is deleted for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment date and time is deleted for music.</t>
-  </si>
-  <si>
     <t>so I can ensure payment confirmation.</t>
   </si>
   <si>
@@ -761,54 +545,12 @@
     <t>Verify order id is created for payment.</t>
   </si>
   <si>
-    <t>Verify payment cost is read for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verify payment cost is read for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment cost is read for music.</t>
-  </si>
-  <si>
-    <t>Verify payment cost is updated for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verify payment cost is updated for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment cost is updated for music.</t>
-  </si>
-  <si>
-    <t>Verify payment cost is deleted for PS4 games.</t>
-  </si>
-  <si>
-    <t>Verify payment cost is deleted for Xbox games.</t>
-  </si>
-  <si>
-    <t>Verfiy payment cost is deleted for music.</t>
-  </si>
-  <si>
-    <t>Verify payment cost is created for PS4 games 0&gt; &amp; &lt;$69.99.</t>
-  </si>
-  <si>
-    <t>Verify payment cost is created for Xbox games 0&gt; &amp; &lt;$69.99.</t>
-  </si>
-  <si>
-    <t>Verfiy payment cost is created for music 0&gt; &amp; &lt;$5.00.</t>
-  </si>
-  <si>
     <t>Verify album title is created 0&gt; &amp; &lt;10.</t>
   </si>
   <si>
-    <t>Verify music title is read.</t>
-  </si>
-  <si>
     <t>Verify music title is updated.</t>
   </si>
   <si>
-    <t>Verify music title is deleted.</t>
-  </si>
-  <si>
     <t>Verify album price is created 0&gt; &amp;  $5.00.</t>
   </si>
   <si>
@@ -821,13 +563,238 @@
     <t>Verify album price is deleted.</t>
   </si>
   <si>
-    <t>Verify purchased PS4 game title is displayed to the customer.</t>
-  </si>
-  <si>
-    <t>Verify purchased Xbox game title is displayed to the customer.</t>
-  </si>
-  <si>
     <t>Verify platform type is displayed to the customer.</t>
+  </si>
+  <si>
+    <t>Verify game title is created.</t>
+  </si>
+  <si>
+    <t>Verify system creates game stock quantity details 0&gt; &amp; &lt;1000.</t>
+  </si>
+  <si>
+    <t>Verify system reads game stock quantity details.</t>
+  </si>
+  <si>
+    <t>Verify system updates game stock quantity details.</t>
+  </si>
+  <si>
+    <t>Verify system deletes game stock quantity details.</t>
+  </si>
+  <si>
+    <t>Verify system prints customer's game.</t>
+  </si>
+  <si>
+    <t>Verify system prints customer's album.</t>
+  </si>
+  <si>
+    <t>Verify album sold cost is displayed.</t>
+  </si>
+  <si>
+    <t>Verify a games sold cost is displayed.</t>
+  </si>
+  <si>
+    <t>Verify purchased game title is displayed to the customer.</t>
+  </si>
+  <si>
+    <t>Verify purchased music title is displayed to the customer.</t>
+  </si>
+  <si>
+    <t>Verify wishlist for a game title is created.</t>
+  </si>
+  <si>
+    <t>Verify wishlist for a game title is read.</t>
+  </si>
+  <si>
+    <t>Verify wishlist for a game title is updated.</t>
+  </si>
+  <si>
+    <t>Verify wishlist for a game title is deleted.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is created for games 0&gt; &amp; &lt;$10.00.</t>
+  </si>
+  <si>
+    <t>Verify album title is read.</t>
+  </si>
+  <si>
+    <t>Verify album title is deleted.</t>
+  </si>
+  <si>
+    <t>Verify artist's name is created 0&gt; &amp; &lt;7.</t>
+  </si>
+  <si>
+    <t>Verify genre is created 0&gt; &amp; &lt;20.</t>
+  </si>
+  <si>
+    <t>Verfiy file url for album is created 0&gt; &amp; &lt;255.</t>
+  </si>
+  <si>
+    <t>Verfiy preview url for album is created 0&gt; &amp; &lt;255.</t>
+  </si>
+  <si>
+    <t>Verify artist's name is read.</t>
+  </si>
+  <si>
+    <t>Verify genre is read.</t>
+  </si>
+  <si>
+    <t>Verfiy file url for album is read.</t>
+  </si>
+  <si>
+    <t>Verfiy preview url for album is read.</t>
+  </si>
+  <si>
+    <t>Verify artist's name is updated.</t>
+  </si>
+  <si>
+    <t>Verify genre is updated.</t>
+  </si>
+  <si>
+    <t>Verfiy file url for album is updated.</t>
+  </si>
+  <si>
+    <t>Verfiy preview url for album is updated.</t>
+  </si>
+  <si>
+    <t>Verify artist's name is deleted.</t>
+  </si>
+  <si>
+    <t>Verify genre is deleted.</t>
+  </si>
+  <si>
+    <t>Verfiy file url for album is deleted.</t>
+  </si>
+  <si>
+    <t>Verfiy preview url for album is deleted.</t>
+  </si>
+  <si>
+    <t>Verify system prints product number.</t>
+  </si>
+  <si>
+    <t>Verify product number is created.</t>
+  </si>
+  <si>
+    <t>I want to create products for stock,</t>
+  </si>
+  <si>
+    <t>so I can sell new products.</t>
+  </si>
+  <si>
+    <t>so I can not sell old products.</t>
+  </si>
+  <si>
+    <t>Verify system creates album stock quantity details 0&gt; &amp; &lt;1000.</t>
+  </si>
+  <si>
+    <t>Verify album title is created.</t>
+  </si>
+  <si>
+    <t>Verify product number is read.</t>
+  </si>
+  <si>
+    <t>Verify album title is updated.</t>
+  </si>
+  <si>
+    <t>Verify product number is updated.</t>
+  </si>
+  <si>
+    <t>Verify product number is deletes.</t>
+  </si>
+  <si>
+    <t>Verify system reads album stock quantity details.</t>
+  </si>
+  <si>
+    <t>Verify system updates album stock quantity details.</t>
+  </si>
+  <si>
+    <t>Verify system deletes album stock quantity details.</t>
+  </si>
+  <si>
+    <t>Verify system prints order number.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is read for games 0&gt; &amp; &lt;$10.00.</t>
+  </si>
+  <si>
+    <t>Verify order id is read for payment.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is created for album 0&gt; &amp; &lt;$5.00.</t>
+  </si>
+  <si>
+    <t>Verify payment status is created for game.</t>
+  </si>
+  <si>
+    <t>Verify payment status is created for album.</t>
+  </si>
+  <si>
+    <t>Verify payment date and time is created for game.</t>
+  </si>
+  <si>
+    <t>Verify payment date and time is created for album.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is read for album 0&gt; &amp; &lt;$5.00.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is updated for games 0&gt; &amp; &lt;$10.00.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is updated for album 0&gt; &amp; &lt;$5.00.</t>
+  </si>
+  <si>
+    <t>Verify order id is updated for payment.</t>
+  </si>
+  <si>
+    <t>Verify payment status is updated for game.</t>
+  </si>
+  <si>
+    <t>Verify payment status is updated for album.</t>
+  </si>
+  <si>
+    <t>Verify payment date and time is updated for game.</t>
+  </si>
+  <si>
+    <t>Verify payment date and time is updated for album.</t>
+  </si>
+  <si>
+    <t>Verify payment cost is deleted for games 0&gt; &amp; &lt;$10.00.</t>
+  </si>
+  <si>
+    <t>Verfiy payment cost is deleted for album 0&gt; &amp; &lt;$5.00.</t>
+  </si>
+  <si>
+    <t>Verify order id is deleted for payment.</t>
+  </si>
+  <si>
+    <t>Verfiy game title is deleted.</t>
+  </si>
+  <si>
+    <t>Verfiy album title is deleted.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is deleted for game.</t>
+  </si>
+  <si>
+    <t>Verfiy payment status is deleted for album.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is deleted for game.</t>
+  </si>
+  <si>
+    <t>Verfiy payment date and time is deleted for album.</t>
+  </si>
+  <si>
+    <t>Verify payment status is read for game.</t>
+  </si>
+  <si>
+    <t>Verify payment status is read for album.</t>
+  </si>
+  <si>
+    <t>Verify payment date and time is read for game.</t>
+  </si>
+  <si>
+    <t>Verify payment date and time is read for album.</t>
   </si>
 </sst>
 </file>
@@ -1270,7 +1237,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62F77FC3-F402-4BE8-8A68-6767566B15A6}">
-  <dimension ref="A1:K247"/>
+  <dimension ref="A1:O251"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -1282,7 +1249,7 @@
       <c r="D1" s="10"/>
       <c r="E1" s="10"/>
       <c r="F1" s="10" t="s">
-        <v>175</v>
+        <v>142</v>
       </c>
       <c r="G1" s="10"/>
       <c r="H1" s="10"/>
@@ -1292,14 +1259,14 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>187</v>
+        <v>154</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
       <c r="E2" s="10"/>
       <c r="F2" s="10" t="s">
-        <v>176</v>
+        <v>143</v>
       </c>
       <c r="G2" s="10"/>
       <c r="H2" s="10"/>
@@ -1309,14 +1276,14 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>173</v>
+        <v>140</v>
       </c>
       <c r="B3" s="10"/>
       <c r="C3" s="10"/>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
       <c r="F3" s="10" t="s">
-        <v>177</v>
+        <v>144</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="10"/>
@@ -1359,7 +1326,7 @@
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
       <c r="F6" s="10" t="s">
-        <v>178</v>
+        <v>145</v>
       </c>
       <c r="G6" s="10"/>
       <c r="H6" s="10"/>
@@ -1369,14 +1336,14 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>188</v>
+        <v>155</v>
       </c>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>
       <c r="F7" s="10" t="s">
-        <v>179</v>
+        <v>146</v>
       </c>
       <c r="G7" s="10"/>
       <c r="H7" s="10"/>
@@ -1386,14 +1353,14 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>174</v>
+        <v>141</v>
       </c>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="10"/>
       <c r="F8" s="10" t="s">
-        <v>180</v>
+        <v>147</v>
       </c>
       <c r="G8" s="10"/>
       <c r="H8" s="10"/>
@@ -1436,7 +1403,7 @@
       <c r="D11" s="10"/>
       <c r="E11" s="10"/>
       <c r="F11" s="10" t="s">
-        <v>181</v>
+        <v>148</v>
       </c>
       <c r="G11" s="10"/>
       <c r="H11" s="10"/>
@@ -1446,14 +1413,14 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>189</v>
+        <v>156</v>
       </c>
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
       <c r="E12" s="10"/>
       <c r="F12" s="10" t="s">
-        <v>182</v>
+        <v>149</v>
       </c>
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
@@ -1463,14 +1430,14 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>191</v>
+        <v>158</v>
       </c>
       <c r="B13" s="10"/>
       <c r="C13" s="10"/>
       <c r="D13" s="10"/>
       <c r="E13" s="10"/>
       <c r="F13" s="10" t="s">
-        <v>183</v>
+        <v>150</v>
       </c>
       <c r="G13" s="10"/>
       <c r="H13" s="10"/>
@@ -1513,7 +1480,7 @@
       <c r="D16" s="10"/>
       <c r="E16" s="10"/>
       <c r="F16" s="10" t="s">
-        <v>184</v>
+        <v>151</v>
       </c>
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
@@ -1523,14 +1490,14 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="10" t="s">
-        <v>190</v>
+        <v>157</v>
       </c>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10"/>
       <c r="E17" s="10"/>
       <c r="F17" s="10" t="s">
-        <v>185</v>
+        <v>152</v>
       </c>
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
@@ -1540,14 +1507,14 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="10" t="s">
-        <v>192</v>
+        <v>159</v>
       </c>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
       <c r="F18" s="10" t="s">
-        <v>186</v>
+        <v>153</v>
       </c>
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
@@ -1594,7 +1561,7 @@
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1" t="s">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
@@ -1611,7 +1578,7 @@
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1" t="s">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
@@ -1626,7 +1593,7 @@
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1" t="s">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>
@@ -1673,7 +1640,7 @@
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1" t="s">
-        <v>68</v>
+        <v>53</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
@@ -1690,7 +1657,7 @@
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="G29" s="1"/>
       <c r="H29" s="1"/>
@@ -1705,7 +1672,7 @@
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1" t="s">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
@@ -1752,7 +1719,7 @@
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="G33" s="1"/>
       <c r="H33" s="1"/>
@@ -1769,7 +1736,7 @@
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
       <c r="F34" s="1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
@@ -1784,7 +1751,7 @@
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
       <c r="F35" s="1" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="G35" s="1"/>
       <c r="H35" s="1"/>
@@ -1831,7 +1798,7 @@
       <c r="D38" s="1"/>
       <c r="E38" s="1"/>
       <c r="F38" s="1" t="s">
-        <v>65</v>
+        <v>50</v>
       </c>
       <c r="G38" s="1"/>
       <c r="H38" s="1"/>
@@ -1848,7 +1815,7 @@
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
       <c r="F39" s="1" t="s">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="G39" s="1"/>
       <c r="H39" s="1"/>
@@ -1863,7 +1830,7 @@
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
       <c r="F40" s="1" t="s">
-        <v>67</v>
+        <v>52</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
@@ -1897,7 +1864,7 @@
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
@@ -1914,7 +1881,7 @@
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
       <c r="F45" s="2" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
@@ -1929,7 +1896,7 @@
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
       <c r="F46" s="2" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
@@ -2183,7 +2150,7 @@
       <c r="D64" s="7"/>
       <c r="E64" s="7"/>
       <c r="F64" s="7" t="s">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="G64" s="7"/>
       <c r="H64" s="7"/>
@@ -2193,14 +2160,14 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="7" t="s">
-        <v>75</v>
+        <v>60</v>
       </c>
       <c r="B65" s="7"/>
       <c r="C65" s="7"/>
       <c r="D65" s="7"/>
       <c r="E65" s="7"/>
       <c r="F65" s="7" t="s">
-        <v>80</v>
+        <v>65</v>
       </c>
       <c r="G65" s="7"/>
       <c r="H65" s="7"/>
@@ -2217,7 +2184,7 @@
       <c r="D66" s="7"/>
       <c r="E66" s="7"/>
       <c r="F66" s="7" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="G66" s="7"/>
       <c r="H66" s="7"/>
@@ -2232,7 +2199,7 @@
       <c r="D67" s="7"/>
       <c r="E67" s="7"/>
       <c r="F67" s="7" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="G67" s="7"/>
       <c r="H67" s="7"/>
@@ -2262,7 +2229,7 @@
       <c r="D69" s="7"/>
       <c r="E69" s="7"/>
       <c r="F69" s="7" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="G69" s="7"/>
       <c r="H69" s="7"/>
@@ -2272,14 +2239,14 @@
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="7" t="s">
-        <v>76</v>
+        <v>61</v>
       </c>
       <c r="B70" s="7"/>
       <c r="C70" s="7"/>
       <c r="D70" s="7"/>
       <c r="E70" s="7"/>
       <c r="F70" s="7" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="G70" s="7"/>
       <c r="H70" s="7"/>
@@ -2296,7 +2263,7 @@
       <c r="D71" s="7"/>
       <c r="E71" s="7"/>
       <c r="F71" s="7" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="G71" s="7"/>
       <c r="H71" s="7"/>
@@ -2311,7 +2278,7 @@
       <c r="D72" s="7"/>
       <c r="E72" s="7"/>
       <c r="F72" s="7" t="s">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="G72" s="7"/>
       <c r="H72" s="7"/>
@@ -2341,7 +2308,7 @@
       <c r="D74" s="7"/>
       <c r="E74" s="7"/>
       <c r="F74" s="7" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="G74" s="7"/>
       <c r="H74" s="7"/>
@@ -2351,14 +2318,14 @@
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="B75" s="7"/>
       <c r="C75" s="7"/>
       <c r="D75" s="7"/>
       <c r="E75" s="7"/>
       <c r="F75" s="7" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="G75" s="7"/>
       <c r="H75" s="7"/>
@@ -2375,7 +2342,7 @@
       <c r="D76" s="7"/>
       <c r="E76" s="7"/>
       <c r="F76" s="7" t="s">
-        <v>89</v>
+        <v>74</v>
       </c>
       <c r="G76" s="7"/>
       <c r="H76" s="7"/>
@@ -2390,7 +2357,7 @@
       <c r="D77" s="7"/>
       <c r="E77" s="7"/>
       <c r="F77" s="7" t="s">
-        <v>90</v>
+        <v>75</v>
       </c>
       <c r="G77" s="7"/>
       <c r="H77" s="7"/>
@@ -2420,7 +2387,7 @@
       <c r="D79" s="7"/>
       <c r="E79" s="7"/>
       <c r="F79" s="7" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="G79" s="7"/>
       <c r="H79" s="7"/>
@@ -2430,14 +2397,14 @@
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" s="7" t="s">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="B80" s="7"/>
       <c r="C80" s="7"/>
       <c r="D80" s="7"/>
       <c r="E80" s="7"/>
       <c r="F80" s="7" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="G80" s="7"/>
       <c r="H80" s="7"/>
@@ -2454,7 +2421,7 @@
       <c r="D81" s="7"/>
       <c r="E81" s="7"/>
       <c r="F81" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="G81" s="7"/>
       <c r="H81" s="7"/>
@@ -2469,7 +2436,7 @@
       <c r="D82" s="7"/>
       <c r="E82" s="7"/>
       <c r="F82" s="7" t="s">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="G82" s="7"/>
       <c r="H82" s="7"/>
@@ -2479,14 +2446,14 @@
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
-        <v>95</v>
+        <v>80</v>
       </c>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
       <c r="D85" s="3"/>
       <c r="E85" s="3"/>
       <c r="F85" s="3" t="s">
-        <v>136</v>
+        <v>111</v>
       </c>
       <c r="G85" s="3"/>
       <c r="H85" s="3"/>
@@ -2496,14 +2463,14 @@
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
       <c r="D86" s="3"/>
       <c r="E86" s="3"/>
       <c r="F86" s="3" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="G86" s="3"/>
       <c r="H86" s="3"/>
@@ -2520,7 +2487,7 @@
       <c r="D87" s="3"/>
       <c r="E87" s="3"/>
       <c r="F87" s="3" t="s">
-        <v>122</v>
+        <v>97</v>
       </c>
       <c r="G87" s="3"/>
       <c r="H87" s="3"/>
@@ -2535,7 +2502,7 @@
       <c r="D88" s="3"/>
       <c r="E88" s="3"/>
       <c r="F88" s="3" t="s">
-        <v>123</v>
+        <v>98</v>
       </c>
       <c r="G88" s="3"/>
       <c r="H88" s="3"/>
@@ -2550,7 +2517,7 @@
       <c r="D89" s="3"/>
       <c r="E89" s="3"/>
       <c r="F89" s="3" t="s">
-        <v>133</v>
+        <v>108</v>
       </c>
       <c r="G89" s="3"/>
       <c r="H89" s="3"/>
@@ -2565,7 +2532,7 @@
       <c r="D90" s="3"/>
       <c r="E90" s="3"/>
       <c r="F90" s="3" t="s">
-        <v>137</v>
+        <v>112</v>
       </c>
       <c r="G90" s="3"/>
       <c r="H90" s="3"/>
@@ -2580,7 +2547,7 @@
       <c r="D91" s="3"/>
       <c r="E91" s="3"/>
       <c r="F91" s="3" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="G91" s="3"/>
       <c r="H91" s="3"/>
@@ -2595,7 +2562,7 @@
       <c r="D92" s="3"/>
       <c r="E92" s="3"/>
       <c r="F92" s="3" t="s">
-        <v>253</v>
+        <v>169</v>
       </c>
       <c r="G92" s="3"/>
       <c r="H92" s="3"/>
@@ -2610,7 +2577,7 @@
       <c r="D93" s="3"/>
       <c r="E93" s="3"/>
       <c r="F93" s="3" t="s">
-        <v>138</v>
+        <v>113</v>
       </c>
       <c r="G93" s="3"/>
       <c r="H93" s="3"/>
@@ -2625,7 +2592,7 @@
       <c r="D94" s="3"/>
       <c r="E94" s="3"/>
       <c r="F94" s="3" t="s">
-        <v>152</v>
+        <v>127</v>
       </c>
       <c r="G94" s="3"/>
       <c r="H94" s="3"/>
@@ -2640,7 +2607,7 @@
       <c r="D95" s="3"/>
       <c r="E95" s="3"/>
       <c r="F95" s="3" t="s">
-        <v>257</v>
+        <v>171</v>
       </c>
       <c r="G95" s="3"/>
       <c r="H95" s="3"/>
@@ -2655,7 +2622,7 @@
       <c r="D96" s="3"/>
       <c r="E96" s="3"/>
       <c r="F96" s="3" t="s">
-        <v>139</v>
+        <v>194</v>
       </c>
       <c r="G96" s="3"/>
       <c r="H96" s="3"/>
@@ -2669,7 +2636,9 @@
       <c r="C97" s="3"/>
       <c r="D97" s="3"/>
       <c r="E97" s="3"/>
-      <c r="F97" s="3"/>
+      <c r="F97" s="3" t="s">
+        <v>195</v>
+      </c>
       <c r="G97" s="3"/>
       <c r="H97" s="3"/>
       <c r="I97" s="3"/>
@@ -2677,15 +2646,13 @@
       <c r="K97" s="3"/>
     </row>
     <row r="98" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A98" s="3" t="s">
-        <v>95</v>
-      </c>
+      <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
       <c r="D98" s="3"/>
       <c r="E98" s="3"/>
       <c r="F98" s="3" t="s">
-        <v>124</v>
+        <v>196</v>
       </c>
       <c r="G98" s="3"/>
       <c r="H98" s="3"/>
@@ -2694,15 +2661,13 @@
       <c r="K98" s="3"/>
     </row>
     <row r="99" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A99" s="3" t="s">
-        <v>72</v>
-      </c>
+      <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
       <c r="D99" s="3"/>
       <c r="E99" s="3"/>
       <c r="F99" s="3" t="s">
-        <v>119</v>
+        <v>197</v>
       </c>
       <c r="G99" s="3"/>
       <c r="H99" s="3"/>
@@ -2711,15 +2676,13 @@
       <c r="K99" s="3"/>
     </row>
     <row r="100" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A100" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
       <c r="D100" s="3"/>
       <c r="E100" s="3"/>
       <c r="F100" s="3" t="s">
-        <v>125</v>
+        <v>114</v>
       </c>
       <c r="G100" s="3"/>
       <c r="H100" s="3"/>
@@ -2733,9 +2696,7 @@
       <c r="C101" s="3"/>
       <c r="D101" s="3"/>
       <c r="E101" s="3"/>
-      <c r="F101" s="3" t="s">
-        <v>126</v>
-      </c>
+      <c r="F101" s="3"/>
       <c r="G101" s="3"/>
       <c r="H101" s="3"/>
       <c r="I101" s="3"/>
@@ -2743,13 +2704,15 @@
       <c r="K101" s="3"/>
     </row>
     <row r="102" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A102" s="3"/>
+      <c r="A102" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
       <c r="D102" s="3"/>
       <c r="E102" s="3"/>
       <c r="F102" s="3" t="s">
-        <v>134</v>
+        <v>99</v>
       </c>
       <c r="G102" s="3"/>
       <c r="H102" s="3"/>
@@ -2758,13 +2721,15 @@
       <c r="K102" s="3"/>
     </row>
     <row r="103" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A103" s="3"/>
+      <c r="A103" s="3" t="s">
+        <v>57</v>
+      </c>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
       <c r="D103" s="3"/>
       <c r="E103" s="3"/>
       <c r="F103" s="3" t="s">
-        <v>140</v>
+        <v>94</v>
       </c>
       <c r="G103" s="3"/>
       <c r="H103" s="3"/>
@@ -2773,13 +2738,15 @@
       <c r="K103" s="3"/>
     </row>
     <row r="104" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A104" s="3"/>
+      <c r="A104" s="3" t="s">
+        <v>19</v>
+      </c>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
       <c r="D104" s="3"/>
       <c r="E104" s="3"/>
       <c r="F104" s="3" t="s">
-        <v>141</v>
+        <v>100</v>
       </c>
       <c r="G104" s="3"/>
       <c r="H104" s="3"/>
@@ -2794,7 +2761,7 @@
       <c r="D105" s="3"/>
       <c r="E105" s="3"/>
       <c r="F105" s="3" t="s">
-        <v>254</v>
+        <v>101</v>
       </c>
       <c r="G105" s="3"/>
       <c r="H105" s="3"/>
@@ -2809,7 +2776,7 @@
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
       <c r="F106" s="3" t="s">
-        <v>142</v>
+        <v>109</v>
       </c>
       <c r="G106" s="3"/>
       <c r="H106" s="3"/>
@@ -2824,7 +2791,7 @@
       <c r="D107" s="3"/>
       <c r="E107" s="3"/>
       <c r="F107" s="3" t="s">
-        <v>154</v>
+        <v>115</v>
       </c>
       <c r="G107" s="3"/>
       <c r="H107" s="3"/>
@@ -2839,7 +2806,7 @@
       <c r="D108" s="3"/>
       <c r="E108" s="3"/>
       <c r="F108" s="3" t="s">
-        <v>258</v>
+        <v>116</v>
       </c>
       <c r="G108" s="3"/>
       <c r="H108" s="3"/>
@@ -2854,7 +2821,7 @@
       <c r="D109" s="3"/>
       <c r="E109" s="3"/>
       <c r="F109" s="3" t="s">
-        <v>143</v>
+        <v>192</v>
       </c>
       <c r="G109" s="3"/>
       <c r="H109" s="3"/>
@@ -2868,7 +2835,9 @@
       <c r="C110" s="3"/>
       <c r="D110" s="3"/>
       <c r="E110" s="3"/>
-      <c r="F110" s="3"/>
+      <c r="F110" s="3" t="s">
+        <v>117</v>
+      </c>
       <c r="G110" s="3"/>
       <c r="H110" s="3"/>
       <c r="I110" s="3"/>
@@ -2876,15 +2845,13 @@
       <c r="K110" s="3"/>
     </row>
     <row r="111" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A111" s="3" t="s">
-        <v>95</v>
-      </c>
+      <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
       <c r="D111" s="3"/>
       <c r="E111" s="3"/>
       <c r="F111" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G111" s="3"/>
       <c r="H111" s="3"/>
@@ -2893,15 +2860,13 @@
       <c r="K111" s="3"/>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A112" s="3" t="s">
-        <v>73</v>
-      </c>
+      <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
       <c r="D112" s="3"/>
       <c r="E112" s="3"/>
       <c r="F112" s="3" t="s">
-        <v>120</v>
+        <v>172</v>
       </c>
       <c r="G112" s="3"/>
       <c r="H112" s="3"/>
@@ -2910,15 +2875,13 @@
       <c r="K112" s="3"/>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A113" s="3" t="s">
-        <v>20</v>
-      </c>
+      <c r="A113" s="3"/>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
       <c r="D113" s="3"/>
       <c r="E113" s="3"/>
       <c r="F113" s="3" t="s">
-        <v>128</v>
+        <v>198</v>
       </c>
       <c r="G113" s="3"/>
       <c r="H113" s="3"/>
@@ -2933,7 +2896,7 @@
       <c r="D114" s="3"/>
       <c r="E114" s="3"/>
       <c r="F114" s="3" t="s">
-        <v>129</v>
+        <v>199</v>
       </c>
       <c r="G114" s="3"/>
       <c r="H114" s="3"/>
@@ -2948,7 +2911,7 @@
       <c r="D115" s="3"/>
       <c r="E115" s="3"/>
       <c r="F115" s="3" t="s">
-        <v>135</v>
+        <v>200</v>
       </c>
       <c r="G115" s="3"/>
       <c r="H115" s="3"/>
@@ -2963,7 +2926,7 @@
       <c r="D116" s="3"/>
       <c r="E116" s="3"/>
       <c r="F116" s="3" t="s">
-        <v>144</v>
+        <v>201</v>
       </c>
       <c r="G116" s="3"/>
       <c r="H116" s="3"/>
@@ -2978,7 +2941,7 @@
       <c r="D117" s="3"/>
       <c r="E117" s="3"/>
       <c r="F117" s="3" t="s">
-        <v>145</v>
+        <v>118</v>
       </c>
       <c r="G117" s="3"/>
       <c r="H117" s="3"/>
@@ -2992,9 +2955,7 @@
       <c r="C118" s="3"/>
       <c r="D118" s="3"/>
       <c r="E118" s="3"/>
-      <c r="F118" s="3" t="s">
-        <v>255</v>
-      </c>
+      <c r="F118" s="3"/>
       <c r="G118" s="3"/>
       <c r="H118" s="3"/>
       <c r="I118" s="3"/>
@@ -3002,13 +2963,15 @@
       <c r="K118" s="3"/>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A119" s="3"/>
+      <c r="A119" s="3" t="s">
+        <v>80</v>
+      </c>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
       <c r="D119" s="3"/>
       <c r="E119" s="3"/>
       <c r="F119" s="3" t="s">
-        <v>146</v>
+        <v>102</v>
       </c>
       <c r="G119" s="3"/>
       <c r="H119" s="3"/>
@@ -3017,13 +2980,15 @@
       <c r="K119" s="3"/>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A120" s="3"/>
+      <c r="A120" s="3" t="s">
+        <v>58</v>
+      </c>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
       <c r="D120" s="3"/>
       <c r="E120" s="3"/>
       <c r="F120" s="3" t="s">
-        <v>155</v>
+        <v>95</v>
       </c>
       <c r="G120" s="3"/>
       <c r="H120" s="3"/>
@@ -3032,13 +2997,15 @@
       <c r="K120" s="3"/>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A121" s="3"/>
+      <c r="A121" s="3" t="s">
+        <v>20</v>
+      </c>
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
       <c r="D121" s="3"/>
       <c r="E121" s="3"/>
       <c r="F121" s="3" t="s">
-        <v>259</v>
+        <v>103</v>
       </c>
       <c r="G121" s="3"/>
       <c r="H121" s="3"/>
@@ -3053,7 +3020,7 @@
       <c r="D122" s="3"/>
       <c r="E122" s="3"/>
       <c r="F122" s="3" t="s">
-        <v>147</v>
+        <v>104</v>
       </c>
       <c r="G122" s="3"/>
       <c r="H122" s="3"/>
@@ -3067,7 +3034,9 @@
       <c r="C123" s="3"/>
       <c r="D123" s="3"/>
       <c r="E123" s="3"/>
-      <c r="F123" s="3"/>
+      <c r="F123" s="3" t="s">
+        <v>110</v>
+      </c>
       <c r="G123" s="3"/>
       <c r="H123" s="3"/>
       <c r="I123" s="3"/>
@@ -3075,15 +3044,13 @@
       <c r="K123" s="3"/>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A124" s="3" t="s">
-        <v>95</v>
-      </c>
+      <c r="A124" s="3"/>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
       <c r="D124" s="3"/>
       <c r="E124" s="3"/>
       <c r="F124" s="3" t="s">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="G124" s="3"/>
       <c r="H124" s="3"/>
@@ -3092,15 +3059,13 @@
       <c r="K124" s="3"/>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A125" s="3" t="s">
-        <v>74</v>
-      </c>
+      <c r="A125" s="3"/>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
       <c r="D125" s="3"/>
       <c r="E125" s="3"/>
       <c r="F125" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G125" s="3"/>
       <c r="H125" s="3"/>
@@ -3109,15 +3074,13 @@
       <c r="K125" s="3"/>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A126" s="3" t="s">
-        <v>21</v>
-      </c>
+      <c r="A126" s="3"/>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
       <c r="D126" s="3"/>
       <c r="E126" s="3"/>
       <c r="F126" s="3" t="s">
-        <v>131</v>
+        <v>170</v>
       </c>
       <c r="G126" s="3"/>
       <c r="H126" s="3"/>
@@ -3132,7 +3095,7 @@
       <c r="D127" s="3"/>
       <c r="E127" s="3"/>
       <c r="F127" s="3" t="s">
-        <v>132</v>
+        <v>121</v>
       </c>
       <c r="G127" s="3"/>
       <c r="H127" s="3"/>
@@ -3147,7 +3110,7 @@
       <c r="D128" s="3"/>
       <c r="E128" s="3"/>
       <c r="F128" s="3" t="s">
-        <v>22</v>
+        <v>130</v>
       </c>
       <c r="G128" s="3"/>
       <c r="H128" s="3"/>
@@ -3155,14 +3118,14 @@
       <c r="J128" s="3"/>
       <c r="K128" s="3"/>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
       <c r="D129" s="3"/>
       <c r="E129" s="3"/>
       <c r="F129" s="3" t="s">
-        <v>148</v>
+        <v>173</v>
       </c>
       <c r="G129" s="3"/>
       <c r="H129" s="3"/>
@@ -3170,14 +3133,14 @@
       <c r="J129" s="3"/>
       <c r="K129" s="3"/>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
       <c r="D130" s="3"/>
       <c r="E130" s="3"/>
       <c r="F130" s="3" t="s">
-        <v>149</v>
+        <v>202</v>
       </c>
       <c r="G130" s="3"/>
       <c r="H130" s="3"/>
@@ -3185,14 +3148,14 @@
       <c r="J130" s="3"/>
       <c r="K130" s="3"/>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
       <c r="D131" s="3"/>
       <c r="E131" s="3"/>
       <c r="F131" s="3" t="s">
-        <v>256</v>
+        <v>203</v>
       </c>
       <c r="G131" s="3"/>
       <c r="H131" s="3"/>
@@ -3200,14 +3163,14 @@
       <c r="J131" s="3"/>
       <c r="K131" s="3"/>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
       <c r="D132" s="3"/>
       <c r="E132" s="3"/>
       <c r="F132" s="3" t="s">
-        <v>150</v>
+        <v>204</v>
       </c>
       <c r="G132" s="3"/>
       <c r="H132" s="3"/>
@@ -3215,14 +3178,14 @@
       <c r="J132" s="3"/>
       <c r="K132" s="3"/>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
       <c r="D133" s="3"/>
       <c r="E133" s="3"/>
       <c r="F133" s="3" t="s">
-        <v>156</v>
+        <v>205</v>
       </c>
       <c r="G133" s="3"/>
       <c r="H133" s="3"/>
@@ -3230,14 +3193,14 @@
       <c r="J133" s="3"/>
       <c r="K133" s="3"/>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
       <c r="D134" s="3"/>
       <c r="E134" s="3"/>
       <c r="F134" s="3" t="s">
-        <v>260</v>
+        <v>122</v>
       </c>
       <c r="G134" s="3"/>
       <c r="H134" s="3"/>
@@ -3245,411 +3208,390 @@
       <c r="J134" s="3"/>
       <c r="K134" s="3"/>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
       <c r="D135" s="3"/>
       <c r="E135" s="3"/>
-      <c r="F135" s="3" t="s">
-        <v>151</v>
-      </c>
+      <c r="F135" s="3"/>
       <c r="G135" s="3"/>
       <c r="H135" s="3"/>
       <c r="I135" s="3"/>
       <c r="J135" s="3"/>
       <c r="K135" s="3"/>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A136" s="11"/>
-      <c r="B136" s="11"/>
-      <c r="C136" s="11"/>
-      <c r="D136" s="11"/>
-      <c r="E136" s="11"/>
-      <c r="F136" s="11"/>
-      <c r="G136" s="11"/>
-      <c r="H136" s="11"/>
-      <c r="I136" s="11"/>
-      <c r="J136" s="11"/>
-      <c r="K136" s="11"/>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A138" s="4" t="s">
+    <row r="136" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A136" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B136" s="3"/>
+      <c r="C136" s="3"/>
+      <c r="D136" s="3"/>
+      <c r="E136" s="3"/>
+      <c r="F136" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="G136" s="3"/>
+      <c r="H136" s="3"/>
+      <c r="I136" s="3"/>
+      <c r="J136" s="3"/>
+      <c r="K136" s="3"/>
+    </row>
+    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A137" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B137" s="3"/>
+      <c r="C137" s="3"/>
+      <c r="D137" s="3"/>
+      <c r="E137" s="3"/>
+      <c r="F137" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="G137" s="3"/>
+      <c r="H137" s="3"/>
+      <c r="I137" s="3"/>
+      <c r="J137" s="3"/>
+      <c r="K137" s="3"/>
+    </row>
+    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A138" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B138" s="3"/>
+      <c r="C138" s="3"/>
+      <c r="D138" s="3"/>
+      <c r="E138" s="3"/>
+      <c r="F138" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G138" s="3"/>
+      <c r="H138" s="3"/>
+      <c r="I138" s="3"/>
+      <c r="J138" s="3"/>
+      <c r="K138" s="3"/>
+    </row>
+    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A139" s="3"/>
+      <c r="B139" s="3"/>
+      <c r="C139" s="3"/>
+      <c r="D139" s="3"/>
+      <c r="E139" s="3"/>
+      <c r="F139" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="G139" s="3"/>
+      <c r="H139" s="3"/>
+      <c r="I139" s="3"/>
+      <c r="J139" s="3"/>
+      <c r="K139" s="3"/>
+    </row>
+    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A140" s="3"/>
+      <c r="B140" s="3"/>
+      <c r="C140" s="3"/>
+      <c r="D140" s="3"/>
+      <c r="E140" s="3"/>
+      <c r="F140" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="G140" s="3"/>
+      <c r="H140" s="3"/>
+      <c r="I140" s="3"/>
+      <c r="J140" s="3"/>
+      <c r="K140" s="3"/>
+    </row>
+    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A141" s="3"/>
+      <c r="B141" s="3"/>
+      <c r="C141" s="3"/>
+      <c r="D141" s="3"/>
+      <c r="E141" s="3"/>
+      <c r="F141" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="G141" s="3"/>
+      <c r="H141" s="3"/>
+      <c r="I141" s="3"/>
+      <c r="J141" s="3"/>
+      <c r="K141" s="3"/>
+    </row>
+    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A142" s="3"/>
+      <c r="B142" s="3"/>
+      <c r="C142" s="3"/>
+      <c r="D142" s="3"/>
+      <c r="E142" s="3"/>
+      <c r="F142" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="G142" s="3"/>
+      <c r="H142" s="3"/>
+      <c r="I142" s="3"/>
+      <c r="J142" s="3"/>
+      <c r="K142" s="3"/>
+      <c r="L142" s="11"/>
+      <c r="M142" s="11"/>
+      <c r="N142" s="11"/>
+      <c r="O142" s="11"/>
+    </row>
+    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A143" s="3"/>
+      <c r="B143" s="3"/>
+      <c r="C143" s="3"/>
+      <c r="D143" s="3"/>
+      <c r="E143" s="3"/>
+      <c r="F143" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G143" s="3"/>
+      <c r="H143" s="3"/>
+      <c r="I143" s="3"/>
+      <c r="J143" s="3"/>
+      <c r="K143" s="3"/>
+    </row>
+    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A144" s="3"/>
+      <c r="B144" s="3"/>
+      <c r="C144" s="3"/>
+      <c r="D144" s="3"/>
+      <c r="E144" s="3"/>
+      <c r="F144" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="G144" s="3"/>
+      <c r="H144" s="3"/>
+      <c r="I144" s="3"/>
+      <c r="J144" s="3"/>
+      <c r="K144" s="3"/>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A145" s="3"/>
+      <c r="B145" s="3"/>
+      <c r="C145" s="3"/>
+      <c r="D145" s="3"/>
+      <c r="E145" s="3"/>
+      <c r="F145" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="G145" s="3"/>
+      <c r="H145" s="3"/>
+      <c r="I145" s="3"/>
+      <c r="J145" s="3"/>
+      <c r="K145" s="3"/>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A146" s="3"/>
+      <c r="B146" s="3"/>
+      <c r="C146" s="3"/>
+      <c r="D146" s="3"/>
+      <c r="E146" s="3"/>
+      <c r="F146" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="G146" s="3"/>
+      <c r="H146" s="3"/>
+      <c r="I146" s="3"/>
+      <c r="J146" s="3"/>
+      <c r="K146" s="3"/>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A147" s="3"/>
+      <c r="B147" s="3"/>
+      <c r="C147" s="3"/>
+      <c r="D147" s="3"/>
+      <c r="E147" s="3"/>
+      <c r="F147" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="G147" s="3"/>
+      <c r="H147" s="3"/>
+      <c r="I147" s="3"/>
+      <c r="J147" s="3"/>
+      <c r="K147" s="3"/>
+    </row>
+    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A148" s="3"/>
+      <c r="B148" s="3"/>
+      <c r="C148" s="3"/>
+      <c r="D148" s="3"/>
+      <c r="E148" s="3"/>
+      <c r="F148" s="3" t="s">
+        <v>207</v>
+      </c>
+      <c r="G148" s="3"/>
+      <c r="H148" s="3"/>
+      <c r="I148" s="3"/>
+      <c r="J148" s="3"/>
+      <c r="K148" s="3"/>
+    </row>
+    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A149" s="3"/>
+      <c r="B149" s="3"/>
+      <c r="C149" s="3"/>
+      <c r="D149" s="3"/>
+      <c r="E149" s="3"/>
+      <c r="F149" s="3" t="s">
+        <v>208</v>
+      </c>
+      <c r="G149" s="3"/>
+      <c r="H149" s="3"/>
+      <c r="I149" s="3"/>
+      <c r="J149" s="3"/>
+      <c r="K149" s="3"/>
+    </row>
+    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A150" s="3"/>
+      <c r="B150" s="3"/>
+      <c r="C150" s="3"/>
+      <c r="D150" s="3"/>
+      <c r="E150" s="3"/>
+      <c r="F150" s="3" t="s">
+        <v>209</v>
+      </c>
+      <c r="G150" s="3"/>
+      <c r="H150" s="3"/>
+      <c r="I150" s="3"/>
+      <c r="J150" s="3"/>
+      <c r="K150" s="3"/>
+    </row>
+    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A151" s="3"/>
+      <c r="B151" s="3"/>
+      <c r="C151" s="3"/>
+      <c r="D151" s="3"/>
+      <c r="E151" s="3"/>
+      <c r="F151" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G151" s="3"/>
+      <c r="H151" s="3"/>
+      <c r="I151" s="3"/>
+      <c r="J151" s="3"/>
+      <c r="K151" s="3"/>
+    </row>
+    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A154" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B138" s="4"/>
-      <c r="C138" s="4"/>
-      <c r="D138" s="4"/>
-      <c r="E138" s="4"/>
-      <c r="F138" s="4" t="s">
-        <v>167</v>
-      </c>
-      <c r="G138" s="4"/>
-      <c r="H138" s="4"/>
-      <c r="I138" s="4"/>
-      <c r="J138" s="4"/>
-      <c r="K138" s="4"/>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A139" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="B139" s="4"/>
-      <c r="C139" s="4"/>
-      <c r="D139" s="4"/>
-      <c r="E139" s="4"/>
-      <c r="F139" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G139" s="4"/>
-      <c r="H139" s="4"/>
-      <c r="I139" s="4"/>
-      <c r="J139" s="4"/>
-      <c r="K139" s="4"/>
-    </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A140" s="4" t="s">
+      <c r="B154" s="4"/>
+      <c r="C154" s="4"/>
+      <c r="D154" s="4"/>
+      <c r="E154" s="4"/>
+      <c r="F154" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="G154" s="4"/>
+      <c r="H154" s="4"/>
+      <c r="I154" s="4"/>
+      <c r="J154" s="4"/>
+      <c r="K154" s="4"/>
+    </row>
+    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A155" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B155" s="4"/>
+      <c r="C155" s="4"/>
+      <c r="D155" s="4"/>
+      <c r="E155" s="4"/>
+      <c r="F155" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="G155" s="4"/>
+      <c r="H155" s="4"/>
+      <c r="I155" s="4"/>
+      <c r="J155" s="4"/>
+      <c r="K155" s="4"/>
+    </row>
+    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A156" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B140" s="4"/>
-      <c r="C140" s="4"/>
-      <c r="D140" s="4"/>
-      <c r="E140" s="4"/>
-      <c r="F140" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="G140" s="4"/>
-      <c r="H140" s="4"/>
-      <c r="I140" s="4"/>
-      <c r="J140" s="4"/>
-      <c r="K140" s="4"/>
-    </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A141" s="4"/>
-      <c r="B141" s="4"/>
-      <c r="C141" s="4"/>
-      <c r="D141" s="4"/>
-      <c r="E141" s="4"/>
-      <c r="F141" s="4" t="s">
+      <c r="B156" s="4"/>
+      <c r="C156" s="4"/>
+      <c r="D156" s="4"/>
+      <c r="E156" s="4"/>
+      <c r="F156" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="G156" s="4"/>
+      <c r="H156" s="4"/>
+      <c r="I156" s="4"/>
+      <c r="J156" s="4"/>
+      <c r="K156" s="4"/>
+    </row>
+    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A157" s="4"/>
+      <c r="B157" s="4"/>
+      <c r="C157" s="4"/>
+      <c r="D157" s="4"/>
+      <c r="E157" s="4"/>
+      <c r="F157" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="G141" s="4"/>
-      <c r="H141" s="4"/>
-      <c r="I141" s="4"/>
-      <c r="J141" s="4"/>
-      <c r="K141" s="4"/>
-    </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A142" s="4"/>
-      <c r="B142" s="4"/>
-      <c r="C142" s="4"/>
-      <c r="D142" s="4"/>
-      <c r="E142" s="4"/>
-      <c r="F142" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="G142" s="4"/>
-      <c r="H142" s="4"/>
-      <c r="I142" s="4"/>
-      <c r="J142" s="4"/>
-      <c r="K142" s="4"/>
-    </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A143" s="4"/>
-      <c r="B143" s="4"/>
-      <c r="C143" s="4"/>
-      <c r="D143" s="4"/>
-      <c r="E143" s="4"/>
-      <c r="F143" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="G143" s="4"/>
-      <c r="H143" s="4"/>
-      <c r="I143" s="4"/>
-      <c r="J143" s="4"/>
-      <c r="K143" s="4"/>
-    </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A145" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B145" s="5"/>
-      <c r="C145" s="5"/>
-      <c r="D145" s="5"/>
-      <c r="E145" s="5"/>
-      <c r="F145" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="G145" s="5"/>
-      <c r="H145" s="5"/>
-      <c r="I145" s="5"/>
-      <c r="J145" s="5"/>
-      <c r="K145" s="5"/>
-    </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A146" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B146" s="5"/>
-      <c r="C146" s="5"/>
-      <c r="D146" s="5"/>
-      <c r="E146" s="5"/>
-      <c r="F146" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="G146" s="5"/>
-      <c r="H146" s="5"/>
-      <c r="I146" s="5"/>
-      <c r="J146" s="5"/>
-      <c r="K146" s="5"/>
-    </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A147" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="B147" s="5"/>
-      <c r="C147" s="5"/>
-      <c r="D147" s="5"/>
-      <c r="E147" s="5"/>
-      <c r="F147" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="G147" s="5"/>
-      <c r="H147" s="5"/>
-      <c r="I147" s="5"/>
-      <c r="J147" s="5"/>
-      <c r="K147" s="5"/>
-    </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A148" s="5"/>
-      <c r="B148" s="5"/>
-      <c r="C148" s="5"/>
-      <c r="D148" s="5"/>
-      <c r="E148" s="5"/>
-      <c r="F148" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G148" s="5"/>
-      <c r="H148" s="5"/>
-      <c r="I148" s="5"/>
-      <c r="J148" s="5"/>
-      <c r="K148" s="5"/>
-    </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A149" s="5"/>
-      <c r="B149" s="5"/>
-      <c r="C149" s="5"/>
-      <c r="D149" s="5"/>
-      <c r="E149" s="5"/>
-      <c r="F149" s="5"/>
-      <c r="G149" s="5"/>
-      <c r="H149" s="5"/>
-      <c r="I149" s="5"/>
-      <c r="J149" s="5"/>
-      <c r="K149" s="5"/>
-    </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A150" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B150" s="5"/>
-      <c r="C150" s="5"/>
-      <c r="D150" s="5"/>
-      <c r="E150" s="5"/>
-      <c r="F150" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="G150" s="5"/>
-      <c r="H150" s="5"/>
-      <c r="I150" s="5"/>
-      <c r="J150" s="5"/>
-      <c r="K150" s="5"/>
-    </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A151" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="B151" s="5"/>
-      <c r="C151" s="5"/>
-      <c r="D151" s="5"/>
-      <c r="E151" s="5"/>
-      <c r="F151" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="G151" s="5"/>
-      <c r="H151" s="5"/>
-      <c r="I151" s="5"/>
-      <c r="J151" s="5"/>
-      <c r="K151" s="5"/>
-    </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A152" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="B152" s="5"/>
-      <c r="C152" s="5"/>
-      <c r="D152" s="5"/>
-      <c r="E152" s="5"/>
-      <c r="F152" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G152" s="5"/>
-      <c r="H152" s="5"/>
-      <c r="I152" s="5"/>
-      <c r="J152" s="5"/>
-      <c r="K152" s="5"/>
-    </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A153" s="5"/>
-      <c r="B153" s="5"/>
-      <c r="C153" s="5"/>
-      <c r="D153" s="5"/>
-      <c r="E153" s="5"/>
-      <c r="F153" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="G153" s="5"/>
-      <c r="H153" s="5"/>
-      <c r="I153" s="5"/>
-      <c r="J153" s="5"/>
-      <c r="K153" s="5"/>
-    </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A154" s="5"/>
-      <c r="B154" s="5"/>
-      <c r="C154" s="5"/>
-      <c r="D154" s="5"/>
-      <c r="E154" s="5"/>
-      <c r="F154" s="5"/>
-      <c r="G154" s="5"/>
-      <c r="H154" s="5"/>
-      <c r="I154" s="5"/>
-      <c r="J154" s="5"/>
-      <c r="K154" s="5"/>
-    </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A155" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B155" s="5"/>
-      <c r="C155" s="5"/>
-      <c r="D155" s="5"/>
-      <c r="E155" s="5"/>
-      <c r="F155" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="G155" s="5"/>
-      <c r="H155" s="5"/>
-      <c r="I155" s="5"/>
-      <c r="J155" s="5"/>
-      <c r="K155" s="5"/>
-    </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A156" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="B156" s="5"/>
-      <c r="C156" s="5"/>
-      <c r="D156" s="5"/>
-      <c r="E156" s="5"/>
-      <c r="F156" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="G156" s="5"/>
-      <c r="H156" s="5"/>
-      <c r="I156" s="5"/>
-      <c r="J156" s="5"/>
-      <c r="K156" s="5"/>
-    </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A157" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B157" s="5"/>
-      <c r="C157" s="5"/>
-      <c r="D157" s="5"/>
-      <c r="E157" s="5"/>
-      <c r="F157" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G157" s="5"/>
-      <c r="H157" s="5"/>
-      <c r="I157" s="5"/>
-      <c r="J157" s="5"/>
-      <c r="K157" s="5"/>
+      <c r="G157" s="4"/>
+      <c r="H157" s="4"/>
+      <c r="I157" s="4"/>
+      <c r="J157" s="4"/>
+      <c r="K157" s="4"/>
     </row>
     <row r="158" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A158" s="5"/>
-      <c r="B158" s="5"/>
-      <c r="C158" s="5"/>
-      <c r="D158" s="5"/>
-      <c r="E158" s="5"/>
-      <c r="F158" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="G158" s="5"/>
-      <c r="H158" s="5"/>
-      <c r="I158" s="5"/>
-      <c r="J158" s="5"/>
-      <c r="K158" s="5"/>
+      <c r="A158" s="4"/>
+      <c r="B158" s="4"/>
+      <c r="C158" s="4"/>
+      <c r="D158" s="4"/>
+      <c r="E158" s="4"/>
+      <c r="F158" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="G158" s="4"/>
+      <c r="H158" s="4"/>
+      <c r="I158" s="4"/>
+      <c r="J158" s="4"/>
+      <c r="K158" s="4"/>
     </row>
     <row r="159" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A159" s="5"/>
-      <c r="B159" s="5"/>
-      <c r="C159" s="5"/>
-      <c r="D159" s="5"/>
-      <c r="E159" s="5"/>
-      <c r="F159" s="5"/>
-      <c r="G159" s="5"/>
-      <c r="H159" s="5"/>
-      <c r="I159" s="5"/>
-      <c r="J159" s="5"/>
-      <c r="K159" s="5"/>
+      <c r="A159" s="4"/>
+      <c r="B159" s="4"/>
+      <c r="C159" s="4"/>
+      <c r="D159" s="4"/>
+      <c r="E159" s="4"/>
+      <c r="F159" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="G159" s="4"/>
+      <c r="H159" s="4"/>
+      <c r="I159" s="4"/>
+      <c r="J159" s="4"/>
+      <c r="K159" s="4"/>
     </row>
     <row r="160" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A160" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="B160" s="5"/>
-      <c r="C160" s="5"/>
-      <c r="D160" s="5"/>
-      <c r="E160" s="5"/>
-      <c r="F160" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="G160" s="5"/>
-      <c r="H160" s="5"/>
-      <c r="I160" s="5"/>
-      <c r="J160" s="5"/>
-      <c r="K160" s="5"/>
-    </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A161" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B161" s="5"/>
-      <c r="C161" s="5"/>
-      <c r="D161" s="5"/>
-      <c r="E161" s="5"/>
-      <c r="F161" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="G161" s="5"/>
-      <c r="H161" s="5"/>
-      <c r="I161" s="5"/>
-      <c r="J161" s="5"/>
-      <c r="K161" s="5"/>
+      <c r="A160" s="4"/>
+      <c r="B160" s="4"/>
+      <c r="C160" s="4"/>
+      <c r="D160" s="4"/>
+      <c r="E160" s="4"/>
+      <c r="F160" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="G160" s="4"/>
+      <c r="H160" s="4"/>
+      <c r="I160" s="4"/>
+      <c r="J160" s="4"/>
+      <c r="K160" s="4"/>
     </row>
     <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162" s="5" t="s">
-        <v>45</v>
+        <v>13</v>
       </c>
       <c r="B162" s="5"/>
       <c r="C162" s="5"/>
       <c r="D162" s="5"/>
       <c r="E162" s="5"/>
       <c r="F162" s="5" t="s">
-        <v>60</v>
+        <v>176</v>
       </c>
       <c r="G162" s="5"/>
       <c r="H162" s="5"/>
@@ -3658,13 +3600,15 @@
       <c r="K162" s="5"/>
     </row>
     <row r="163" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A163" s="5"/>
+      <c r="A163" s="5" t="s">
+        <v>212</v>
+      </c>
       <c r="B163" s="5"/>
       <c r="C163" s="5"/>
       <c r="D163" s="5"/>
       <c r="E163" s="5"/>
       <c r="F163" s="5" t="s">
-        <v>61</v>
+        <v>216</v>
       </c>
       <c r="G163" s="5"/>
       <c r="H163" s="5"/>
@@ -3673,711 +3617,709 @@
       <c r="K163" s="5"/>
     </row>
     <row r="164" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A164" s="5"/>
+      <c r="A164" s="5" t="s">
+        <v>38</v>
+      </c>
       <c r="B164" s="5"/>
       <c r="C164" s="5"/>
       <c r="D164" s="5"/>
       <c r="E164" s="5"/>
-      <c r="F164" s="5"/>
+      <c r="F164" s="5" t="s">
+        <v>215</v>
+      </c>
       <c r="G164" s="5"/>
       <c r="H164" s="5"/>
       <c r="I164" s="5"/>
       <c r="J164" s="5"/>
       <c r="K164" s="5"/>
     </row>
+    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A165" s="5"/>
+      <c r="B165" s="5"/>
+      <c r="C165" s="5"/>
+      <c r="D165" s="5"/>
+      <c r="E165" s="5"/>
+      <c r="F165" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="G165" s="5"/>
+      <c r="H165" s="5"/>
+      <c r="I165" s="5"/>
+      <c r="J165" s="5"/>
+      <c r="K165" s="5"/>
+    </row>
+    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A166" s="5"/>
+      <c r="B166" s="5"/>
+      <c r="C166" s="5"/>
+      <c r="D166" s="5"/>
+      <c r="E166" s="5"/>
+      <c r="F166" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="G166" s="5"/>
+      <c r="H166" s="5"/>
+      <c r="I166" s="5"/>
+      <c r="J166" s="5"/>
+      <c r="K166" s="5"/>
+    </row>
     <row r="167" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A167" s="6" t="s">
+      <c r="A167" s="5"/>
+      <c r="B167" s="5"/>
+      <c r="C167" s="5"/>
+      <c r="D167" s="5"/>
+      <c r="E167" s="5"/>
+      <c r="F167" s="5"/>
+      <c r="G167" s="5"/>
+      <c r="H167" s="5"/>
+      <c r="I167" s="5"/>
+      <c r="J167" s="5"/>
+      <c r="K167" s="5"/>
+    </row>
+    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A168" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B167" s="6"/>
-      <c r="C167" s="6"/>
-      <c r="D167" s="6"/>
-      <c r="E167" s="6"/>
-      <c r="F167" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="G167" s="6"/>
-      <c r="H167" s="6"/>
-      <c r="I167" s="6"/>
-      <c r="J167" s="6"/>
-      <c r="K167" s="6"/>
-    </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A168" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="B168" s="6"/>
-      <c r="C168" s="6"/>
-      <c r="D168" s="6"/>
-      <c r="E168" s="6"/>
-      <c r="F168" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="G168" s="6"/>
-      <c r="H168" s="6"/>
-      <c r="I168" s="6"/>
-      <c r="J168" s="6"/>
-      <c r="K168" s="6"/>
+      <c r="B168" s="5"/>
+      <c r="C168" s="5"/>
+      <c r="D168" s="5"/>
+      <c r="E168" s="5"/>
+      <c r="F168" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="G168" s="5"/>
+      <c r="H168" s="5"/>
+      <c r="I168" s="5"/>
+      <c r="J168" s="5"/>
+      <c r="K168" s="5"/>
     </row>
     <row r="169" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A169" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="B169" s="6"/>
-      <c r="C169" s="6"/>
-      <c r="D169" s="6"/>
-      <c r="E169" s="6"/>
-      <c r="F169" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="G169" s="6"/>
-      <c r="H169" s="6"/>
-      <c r="I169" s="6"/>
-      <c r="J169" s="6"/>
-      <c r="K169" s="6"/>
+      <c r="A169" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B169" s="5"/>
+      <c r="C169" s="5"/>
+      <c r="D169" s="5"/>
+      <c r="E169" s="5"/>
+      <c r="F169" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="G169" s="5"/>
+      <c r="H169" s="5"/>
+      <c r="I169" s="5"/>
+      <c r="J169" s="5"/>
+      <c r="K169" s="5"/>
     </row>
     <row r="170" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A170" s="6"/>
-      <c r="B170" s="6"/>
-      <c r="C170" s="6"/>
-      <c r="D170" s="6"/>
-      <c r="E170" s="6"/>
-      <c r="F170" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="G170" s="6"/>
-      <c r="H170" s="6"/>
-      <c r="I170" s="6"/>
-      <c r="J170" s="6"/>
-      <c r="K170" s="6"/>
+      <c r="A170" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B170" s="5"/>
+      <c r="C170" s="5"/>
+      <c r="D170" s="5"/>
+      <c r="E170" s="5"/>
+      <c r="F170" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="G170" s="5"/>
+      <c r="H170" s="5"/>
+      <c r="I170" s="5"/>
+      <c r="J170" s="5"/>
+      <c r="K170" s="5"/>
+    </row>
+    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A171" s="5"/>
+      <c r="B171" s="5"/>
+      <c r="C171" s="5"/>
+      <c r="D171" s="5"/>
+      <c r="E171" s="5"/>
+      <c r="F171" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="G171" s="5"/>
+      <c r="H171" s="5"/>
+      <c r="I171" s="5"/>
+      <c r="J171" s="5"/>
+      <c r="K171" s="5"/>
     </row>
     <row r="172" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A172" s="8" t="s">
-        <v>96</v>
-      </c>
-      <c r="B172" s="8"/>
-      <c r="C172" s="8"/>
-      <c r="D172" s="8"/>
-      <c r="E172" s="8" t="s">
-        <v>261</v>
-      </c>
-      <c r="F172" s="8"/>
-      <c r="G172" s="8"/>
-      <c r="H172" s="8"/>
-      <c r="I172" s="8"/>
-      <c r="J172" s="8"/>
-      <c r="K172" s="8"/>
+      <c r="A172" s="5"/>
+      <c r="B172" s="5"/>
+      <c r="C172" s="5"/>
+      <c r="D172" s="5"/>
+      <c r="E172" s="5"/>
+      <c r="F172" s="5" t="s">
+        <v>217</v>
+      </c>
+      <c r="G172" s="5"/>
+      <c r="H172" s="5"/>
+      <c r="I172" s="5"/>
+      <c r="J172" s="5"/>
+      <c r="K172" s="5"/>
     </row>
     <row r="173" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A173" s="8" t="s">
-        <v>97</v>
-      </c>
-      <c r="B173" s="8"/>
-      <c r="C173" s="8"/>
-      <c r="D173" s="8"/>
-      <c r="E173" s="8" t="s">
-        <v>262</v>
-      </c>
-      <c r="F173" s="8"/>
-      <c r="G173" s="8"/>
-      <c r="H173" s="8"/>
-      <c r="I173" s="8"/>
-      <c r="J173" s="8"/>
-      <c r="K173" s="8"/>
+      <c r="A173" s="5"/>
+      <c r="B173" s="5"/>
+      <c r="C173" s="5"/>
+      <c r="D173" s="5"/>
+      <c r="E173" s="5"/>
+      <c r="F173" s="5"/>
+      <c r="G173" s="5"/>
+      <c r="H173" s="5"/>
+      <c r="I173" s="5"/>
+      <c r="J173" s="5"/>
+      <c r="K173" s="5"/>
     </row>
     <row r="174" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A174" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="B174" s="8"/>
-      <c r="C174" s="8"/>
-      <c r="D174" s="8"/>
-      <c r="E174" s="8" t="s">
-        <v>263</v>
-      </c>
-      <c r="F174" s="8"/>
-      <c r="G174" s="8"/>
-      <c r="H174" s="8"/>
-      <c r="I174" s="8"/>
-      <c r="J174" s="8"/>
-      <c r="K174" s="8"/>
+      <c r="A174" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B174" s="5"/>
+      <c r="C174" s="5"/>
+      <c r="D174" s="5"/>
+      <c r="E174" s="5"/>
+      <c r="F174" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="G174" s="5"/>
+      <c r="H174" s="5"/>
+      <c r="I174" s="5"/>
+      <c r="J174" s="5"/>
+      <c r="K174" s="5"/>
     </row>
     <row r="175" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A175" s="8"/>
-      <c r="B175" s="8"/>
-      <c r="C175" s="8"/>
-      <c r="D175" s="8"/>
-      <c r="E175" s="8" t="s">
-        <v>172</v>
-      </c>
-      <c r="F175" s="8"/>
-      <c r="G175" s="8"/>
-      <c r="H175" s="8"/>
-      <c r="I175" s="8"/>
-      <c r="J175" s="8"/>
-      <c r="K175" s="8"/>
+      <c r="A175" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="B175" s="5"/>
+      <c r="C175" s="5"/>
+      <c r="D175" s="5"/>
+      <c r="E175" s="5"/>
+      <c r="F175" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="G175" s="5"/>
+      <c r="H175" s="5"/>
+      <c r="I175" s="5"/>
+      <c r="J175" s="5"/>
+      <c r="K175" s="5"/>
+    </row>
+    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A176" s="5" t="s">
+        <v>213</v>
+      </c>
+      <c r="B176" s="5"/>
+      <c r="C176" s="5"/>
+      <c r="D176" s="5"/>
+      <c r="E176" s="5"/>
+      <c r="F176" s="5" t="s">
+        <v>222</v>
+      </c>
+      <c r="G176" s="5"/>
+      <c r="H176" s="5"/>
+      <c r="I176" s="5"/>
+      <c r="J176" s="5"/>
+      <c r="K176" s="5"/>
     </row>
     <row r="177" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A177" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B177" s="9"/>
-      <c r="C177" s="9"/>
-      <c r="D177" s="9"/>
-      <c r="E177" s="9"/>
-      <c r="F177" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="G177" s="9"/>
-      <c r="H177" s="9"/>
-      <c r="I177" s="9"/>
-      <c r="J177" s="9"/>
-      <c r="K177" s="9"/>
+      <c r="A177" s="5"/>
+      <c r="B177" s="5"/>
+      <c r="C177" s="5"/>
+      <c r="D177" s="5"/>
+      <c r="E177" s="5"/>
+      <c r="F177" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="G177" s="5"/>
+      <c r="H177" s="5"/>
+      <c r="I177" s="5"/>
+      <c r="J177" s="5"/>
+      <c r="K177" s="5"/>
     </row>
     <row r="178" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A178" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="B178" s="9"/>
-      <c r="C178" s="9"/>
-      <c r="D178" s="9"/>
-      <c r="E178" s="9"/>
-      <c r="F178" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="G178" s="9"/>
-      <c r="H178" s="9"/>
-      <c r="I178" s="9"/>
-      <c r="J178" s="9"/>
-      <c r="K178" s="9"/>
+      <c r="A178" s="5"/>
+      <c r="B178" s="5"/>
+      <c r="C178" s="5"/>
+      <c r="D178" s="5"/>
+      <c r="E178" s="5"/>
+      <c r="F178" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="G178" s="5"/>
+      <c r="H178" s="5"/>
+      <c r="I178" s="5"/>
+      <c r="J178" s="5"/>
+      <c r="K178" s="5"/>
     </row>
     <row r="179" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A179" s="9" t="s">
-        <v>117</v>
-      </c>
-      <c r="B179" s="9"/>
-      <c r="C179" s="9"/>
-      <c r="D179" s="9"/>
-      <c r="E179" s="9"/>
-      <c r="F179" s="9" t="s">
-        <v>113</v>
-      </c>
-      <c r="G179" s="9"/>
-      <c r="H179" s="9"/>
-      <c r="I179" s="9"/>
-      <c r="J179" s="9"/>
-      <c r="K179" s="9"/>
+      <c r="A179" s="5"/>
+      <c r="B179" s="5"/>
+      <c r="C179" s="5"/>
+      <c r="D179" s="5"/>
+      <c r="E179" s="5"/>
+      <c r="F179" s="5"/>
+      <c r="G179" s="5"/>
+      <c r="H179" s="5"/>
+      <c r="I179" s="5"/>
+      <c r="J179" s="5"/>
+      <c r="K179" s="5"/>
     </row>
     <row r="180" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A180" s="9"/>
-      <c r="B180" s="9"/>
-      <c r="C180" s="9"/>
-      <c r="D180" s="9"/>
-      <c r="E180" s="9"/>
-      <c r="F180" s="9"/>
-      <c r="G180" s="9"/>
-      <c r="H180" s="9"/>
-      <c r="I180" s="9"/>
-      <c r="J180" s="9"/>
-      <c r="K180" s="9"/>
+      <c r="A180" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="B180" s="5"/>
+      <c r="C180" s="5"/>
+      <c r="D180" s="5"/>
+      <c r="E180" s="5"/>
+      <c r="F180" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="G180" s="5"/>
+      <c r="H180" s="5"/>
+      <c r="I180" s="5"/>
+      <c r="J180" s="5"/>
+      <c r="K180" s="5"/>
     </row>
     <row r="181" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A181" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B181" s="9"/>
-      <c r="C181" s="9"/>
-      <c r="D181" s="9"/>
-      <c r="E181" s="9"/>
-      <c r="F181" s="9" t="s">
-        <v>162</v>
-      </c>
-      <c r="G181" s="9"/>
-      <c r="H181" s="9"/>
-      <c r="I181" s="9"/>
-      <c r="J181" s="9"/>
-      <c r="K181" s="9"/>
+      <c r="A181" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="B181" s="5"/>
+      <c r="C181" s="5"/>
+      <c r="D181" s="5"/>
+      <c r="E181" s="5"/>
+      <c r="F181" s="5" t="s">
+        <v>193</v>
+      </c>
+      <c r="G181" s="5"/>
+      <c r="H181" s="5"/>
+      <c r="I181" s="5"/>
+      <c r="J181" s="5"/>
+      <c r="K181" s="5"/>
     </row>
     <row r="182" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A182" s="9" t="s">
-        <v>106</v>
-      </c>
-      <c r="B182" s="9"/>
-      <c r="C182" s="9"/>
-      <c r="D182" s="9"/>
-      <c r="E182" s="9"/>
-      <c r="F182" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="G182" s="9"/>
-      <c r="H182" s="9"/>
-      <c r="I182" s="9"/>
-      <c r="J182" s="9"/>
-      <c r="K182" s="9"/>
+      <c r="A182" s="5" t="s">
+        <v>214</v>
+      </c>
+      <c r="B182" s="5"/>
+      <c r="C182" s="5"/>
+      <c r="D182" s="5"/>
+      <c r="E182" s="5"/>
+      <c r="F182" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="G182" s="5"/>
+      <c r="H182" s="5"/>
+      <c r="I182" s="5"/>
+      <c r="J182" s="5"/>
+      <c r="K182" s="5"/>
     </row>
     <row r="183" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A183" s="9" t="s">
-        <v>107</v>
-      </c>
-      <c r="B183" s="9"/>
-      <c r="C183" s="9"/>
-      <c r="D183" s="9"/>
-      <c r="E183" s="9"/>
-      <c r="F183" s="9" t="s">
-        <v>114</v>
-      </c>
-      <c r="G183" s="9"/>
-      <c r="H183" s="9"/>
-      <c r="I183" s="9"/>
-      <c r="J183" s="9"/>
-      <c r="K183" s="9"/>
+      <c r="A183" s="5"/>
+      <c r="B183" s="5"/>
+      <c r="C183" s="5"/>
+      <c r="D183" s="5"/>
+      <c r="E183" s="5"/>
+      <c r="F183" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="G183" s="5"/>
+      <c r="H183" s="5"/>
+      <c r="I183" s="5"/>
+      <c r="J183" s="5"/>
+      <c r="K183" s="5"/>
     </row>
     <row r="184" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A184" s="9"/>
-      <c r="B184" s="9"/>
-      <c r="C184" s="9"/>
-      <c r="D184" s="9"/>
-      <c r="E184" s="9"/>
-      <c r="F184" s="9"/>
-      <c r="G184" s="9"/>
-      <c r="H184" s="9"/>
-      <c r="I184" s="9"/>
-      <c r="J184" s="9"/>
-      <c r="K184" s="9"/>
-    </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A185" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B185" s="9"/>
-      <c r="C185" s="9"/>
-      <c r="D185" s="9"/>
-      <c r="E185" s="9"/>
-      <c r="F185" s="9" t="s">
-        <v>163</v>
-      </c>
-      <c r="G185" s="9"/>
-      <c r="H185" s="9"/>
-      <c r="I185" s="9"/>
-      <c r="J185" s="9"/>
-      <c r="K185" s="9"/>
-    </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A186" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="B186" s="9"/>
-      <c r="C186" s="9"/>
-      <c r="D186" s="9"/>
-      <c r="E186" s="9"/>
-      <c r="F186" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="G186" s="9"/>
-      <c r="H186" s="9"/>
-      <c r="I186" s="9"/>
-      <c r="J186" s="9"/>
-      <c r="K186" s="9"/>
+      <c r="A184" s="5"/>
+      <c r="B184" s="5"/>
+      <c r="C184" s="5"/>
+      <c r="D184" s="5"/>
+      <c r="E184" s="5"/>
+      <c r="F184" s="5" t="s">
+        <v>220</v>
+      </c>
+      <c r="G184" s="5"/>
+      <c r="H184" s="5"/>
+      <c r="I184" s="5"/>
+      <c r="J184" s="5"/>
+      <c r="K184" s="5"/>
     </row>
     <row r="187" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A187" s="9" t="s">
-        <v>110</v>
-      </c>
-      <c r="B187" s="9"/>
-      <c r="C187" s="9"/>
-      <c r="D187" s="9"/>
-      <c r="E187" s="9"/>
-      <c r="F187" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="G187" s="9"/>
-      <c r="H187" s="9"/>
-      <c r="I187" s="9"/>
-      <c r="J187" s="9"/>
-      <c r="K187" s="9"/>
+      <c r="A187" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B187" s="6"/>
+      <c r="C187" s="6"/>
+      <c r="D187" s="6"/>
+      <c r="E187" s="6"/>
+      <c r="F187" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="G187" s="6"/>
+      <c r="H187" s="6"/>
+      <c r="I187" s="6"/>
+      <c r="J187" s="6"/>
+      <c r="K187" s="6"/>
     </row>
     <row r="188" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A188" s="9"/>
-      <c r="B188" s="9"/>
-      <c r="C188" s="9"/>
-      <c r="D188" s="9"/>
-      <c r="E188" s="9"/>
-      <c r="F188" s="9"/>
-      <c r="G188" s="9"/>
-      <c r="H188" s="9"/>
-      <c r="I188" s="9"/>
-      <c r="J188" s="9"/>
-      <c r="K188" s="9"/>
+      <c r="A188" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="B188" s="6"/>
+      <c r="C188" s="6"/>
+      <c r="D188" s="6"/>
+      <c r="E188" s="6"/>
+      <c r="F188" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="G188" s="6"/>
+      <c r="H188" s="6"/>
+      <c r="I188" s="6"/>
+      <c r="J188" s="6"/>
+      <c r="K188" s="6"/>
     </row>
     <row r="189" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A189" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="B189" s="9"/>
-      <c r="C189" s="9"/>
-      <c r="D189" s="9"/>
-      <c r="E189" s="9"/>
-      <c r="F189" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="G189" s="9"/>
-      <c r="H189" s="9"/>
-      <c r="I189" s="9"/>
-      <c r="J189" s="9"/>
-      <c r="K189" s="9"/>
+      <c r="A189" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B189" s="6"/>
+      <c r="C189" s="6"/>
+      <c r="D189" s="6"/>
+      <c r="E189" s="6"/>
+      <c r="F189" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="G189" s="6"/>
+      <c r="H189" s="6"/>
+      <c r="I189" s="6"/>
+      <c r="J189" s="6"/>
+      <c r="K189" s="6"/>
     </row>
     <row r="190" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A190" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="B190" s="9"/>
-      <c r="C190" s="9"/>
-      <c r="D190" s="9"/>
-      <c r="E190" s="9"/>
-      <c r="F190" s="9" t="s">
-        <v>105</v>
-      </c>
-      <c r="G190" s="9"/>
-      <c r="H190" s="9"/>
-      <c r="I190" s="9"/>
-      <c r="J190" s="9"/>
-      <c r="K190" s="9"/>
-    </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A191" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="B191" s="9"/>
-      <c r="C191" s="9"/>
-      <c r="D191" s="9"/>
-      <c r="E191" s="9"/>
-      <c r="F191" s="9" t="s">
-        <v>116</v>
-      </c>
-      <c r="G191" s="9"/>
-      <c r="H191" s="9"/>
-      <c r="I191" s="9"/>
-      <c r="J191" s="9"/>
-      <c r="K191" s="9"/>
+      <c r="A190" s="6"/>
+      <c r="B190" s="6"/>
+      <c r="C190" s="6"/>
+      <c r="D190" s="6"/>
+      <c r="E190" s="6"/>
+      <c r="F190" s="6"/>
+      <c r="G190" s="6"/>
+      <c r="H190" s="6"/>
+      <c r="I190" s="6"/>
+      <c r="J190" s="6"/>
+      <c r="K190" s="6"/>
+    </row>
+    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A192" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B192" s="8"/>
+      <c r="C192" s="8"/>
+      <c r="D192" s="8"/>
+      <c r="E192" s="8" t="s">
+        <v>185</v>
+      </c>
+      <c r="F192" s="8"/>
+      <c r="G192" s="8"/>
+      <c r="H192" s="8"/>
+      <c r="I192" s="8"/>
+      <c r="J192" s="8"/>
+      <c r="K192" s="8"/>
     </row>
     <row r="193" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A193" s="4" t="s">
+      <c r="A193" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="B193" s="8"/>
+      <c r="C193" s="8"/>
+      <c r="D193" s="8"/>
+      <c r="E193" s="8" t="s">
+        <v>186</v>
+      </c>
+      <c r="F193" s="8"/>
+      <c r="G193" s="8"/>
+      <c r="H193" s="8"/>
+      <c r="I193" s="8"/>
+      <c r="J193" s="8"/>
+      <c r="K193" s="8"/>
+    </row>
+    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A194" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B194" s="8"/>
+      <c r="C194" s="8"/>
+      <c r="D194" s="8"/>
+      <c r="E194" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="F194" s="8"/>
+      <c r="G194" s="8"/>
+      <c r="H194" s="8"/>
+      <c r="I194" s="8"/>
+      <c r="J194" s="8"/>
+      <c r="K194" s="8"/>
+    </row>
+    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A195" s="8"/>
+      <c r="B195" s="8"/>
+      <c r="C195" s="8"/>
+      <c r="D195" s="8"/>
+      <c r="E195" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="F195" s="8"/>
+      <c r="G195" s="8"/>
+      <c r="H195" s="8"/>
+      <c r="I195" s="8"/>
+      <c r="J195" s="8"/>
+      <c r="K195" s="8"/>
+    </row>
+    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A197" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B197" s="9"/>
+      <c r="C197" s="9"/>
+      <c r="D197" s="9"/>
+      <c r="E197" s="9"/>
+      <c r="F197" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="G197" s="9"/>
+      <c r="H197" s="9"/>
+      <c r="I197" s="9"/>
+      <c r="J197" s="9"/>
+      <c r="K197" s="9"/>
+    </row>
+    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A198" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B198" s="9"/>
+      <c r="C198" s="9"/>
+      <c r="D198" s="9"/>
+      <c r="E198" s="9"/>
+      <c r="F198" s="9" t="s">
+        <v>187</v>
+      </c>
+      <c r="G198" s="9"/>
+      <c r="H198" s="9"/>
+      <c r="I198" s="9"/>
+      <c r="J198" s="9"/>
+      <c r="K198" s="9"/>
+    </row>
+    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A199" s="9" t="s">
+        <v>92</v>
+      </c>
+      <c r="B199" s="9"/>
+      <c r="C199" s="9"/>
+      <c r="D199" s="9"/>
+      <c r="E199" s="9"/>
+      <c r="F199" s="9"/>
+      <c r="G199" s="9"/>
+      <c r="H199" s="9"/>
+      <c r="I199" s="9"/>
+      <c r="J199" s="9"/>
+      <c r="K199" s="9"/>
+    </row>
+    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A200" s="9"/>
+      <c r="B200" s="9"/>
+      <c r="C200" s="9"/>
+      <c r="D200" s="9"/>
+      <c r="E200" s="9"/>
+      <c r="F200" s="9"/>
+      <c r="G200" s="9"/>
+      <c r="H200" s="9"/>
+      <c r="I200" s="9"/>
+      <c r="J200" s="9"/>
+      <c r="K200" s="9"/>
+    </row>
+    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A201" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B201" s="9"/>
+      <c r="C201" s="9"/>
+      <c r="D201" s="9"/>
+      <c r="E201" s="9"/>
+      <c r="F201" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="G201" s="9"/>
+      <c r="H201" s="9"/>
+      <c r="I201" s="9"/>
+      <c r="J201" s="9"/>
+      <c r="K201" s="9"/>
+    </row>
+    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A202" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="B202" s="9"/>
+      <c r="C202" s="9"/>
+      <c r="D202" s="9"/>
+      <c r="E202" s="9"/>
+      <c r="F202" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="G202" s="9"/>
+      <c r="H202" s="9"/>
+      <c r="I202" s="9"/>
+      <c r="J202" s="9"/>
+      <c r="K202" s="9"/>
+    </row>
+    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A203" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="B203" s="9"/>
+      <c r="C203" s="9"/>
+      <c r="D203" s="9"/>
+      <c r="E203" s="9"/>
+      <c r="F203" s="9"/>
+      <c r="G203" s="9"/>
+      <c r="H203" s="9"/>
+      <c r="I203" s="9"/>
+      <c r="J203" s="9"/>
+      <c r="K203" s="9"/>
+    </row>
+    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A204" s="9"/>
+      <c r="B204" s="9"/>
+      <c r="C204" s="9"/>
+      <c r="D204" s="9"/>
+      <c r="E204" s="9"/>
+      <c r="F204" s="9"/>
+      <c r="G204" s="9"/>
+      <c r="H204" s="9"/>
+      <c r="I204" s="9"/>
+      <c r="J204" s="9"/>
+      <c r="K204" s="9"/>
+    </row>
+    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A205" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B205" s="9"/>
+      <c r="C205" s="9"/>
+      <c r="D205" s="9"/>
+      <c r="E205" s="9"/>
+      <c r="F205" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="G205" s="9"/>
+      <c r="H205" s="9"/>
+      <c r="I205" s="9"/>
+      <c r="J205" s="9"/>
+      <c r="K205" s="9"/>
+    </row>
+    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A206" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B206" s="9"/>
+      <c r="C206" s="9"/>
+      <c r="D206" s="9"/>
+      <c r="E206" s="9"/>
+      <c r="F206" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="G206" s="9"/>
+      <c r="H206" s="9"/>
+      <c r="I206" s="9"/>
+      <c r="J206" s="9"/>
+      <c r="K206" s="9"/>
+    </row>
+    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A207" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="B207" s="9"/>
+      <c r="C207" s="9"/>
+      <c r="D207" s="9"/>
+      <c r="E207" s="9"/>
+      <c r="F207" s="9"/>
+      <c r="G207" s="9"/>
+      <c r="H207" s="9"/>
+      <c r="I207" s="9"/>
+      <c r="J207" s="9"/>
+      <c r="K207" s="9"/>
+    </row>
+    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A208" s="9"/>
+      <c r="B208" s="9"/>
+      <c r="C208" s="9"/>
+      <c r="D208" s="9"/>
+      <c r="E208" s="9"/>
+      <c r="F208" s="9"/>
+      <c r="G208" s="9"/>
+      <c r="H208" s="9"/>
+      <c r="I208" s="9"/>
+      <c r="J208" s="9"/>
+      <c r="K208" s="9"/>
+    </row>
+    <row r="209" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A209" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="B209" s="9"/>
+      <c r="C209" s="9"/>
+      <c r="D209" s="9"/>
+      <c r="E209" s="9"/>
+      <c r="F209" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="G209" s="9"/>
+      <c r="H209" s="9"/>
+      <c r="I209" s="9"/>
+      <c r="J209" s="9"/>
+      <c r="K209" s="9"/>
+    </row>
+    <row r="210" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A210" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B210" s="9"/>
+      <c r="C210" s="9"/>
+      <c r="D210" s="9"/>
+      <c r="E210" s="9"/>
+      <c r="F210" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="G210" s="9"/>
+      <c r="H210" s="9"/>
+      <c r="I210" s="9"/>
+      <c r="J210" s="9"/>
+      <c r="K210" s="9"/>
+    </row>
+    <row r="211" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A211" s="9" t="s">
+        <v>90</v>
+      </c>
+      <c r="B211" s="9"/>
+      <c r="C211" s="9"/>
+      <c r="D211" s="9"/>
+      <c r="E211" s="9"/>
+      <c r="F211" s="9"/>
+      <c r="G211" s="9"/>
+      <c r="H211" s="9"/>
+      <c r="I211" s="9"/>
+      <c r="J211" s="9"/>
+      <c r="K211" s="9"/>
+    </row>
+    <row r="213" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A213" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B193" s="4"/>
-      <c r="C193" s="4"/>
-      <c r="D193" s="4"/>
-      <c r="E193" s="4"/>
-      <c r="F193" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="G193" s="4"/>
-      <c r="H193" s="4"/>
-      <c r="I193" s="4"/>
-      <c r="J193" s="4"/>
-      <c r="K193" s="4"/>
-    </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A194" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="B194" s="4"/>
-      <c r="C194" s="4"/>
-      <c r="D194" s="4"/>
-      <c r="E194" s="4"/>
-      <c r="F194" s="4" t="s">
-        <v>251</v>
-      </c>
-      <c r="G194" s="4"/>
-      <c r="H194" s="4"/>
-      <c r="I194" s="4"/>
-      <c r="J194" s="4"/>
-      <c r="K194" s="4"/>
-    </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A195" s="4" t="s">
-        <v>193</v>
-      </c>
-      <c r="B195" s="4"/>
-      <c r="C195" s="4"/>
-      <c r="D195" s="4"/>
-      <c r="E195" s="4"/>
-      <c r="F195" s="4" t="s">
-        <v>252</v>
-      </c>
-      <c r="G195" s="4"/>
-      <c r="H195" s="4"/>
-      <c r="I195" s="4"/>
-      <c r="J195" s="4"/>
-      <c r="K195" s="4"/>
-    </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A196" s="4"/>
-      <c r="B196" s="4"/>
-      <c r="C196" s="4"/>
-      <c r="D196" s="4"/>
-      <c r="E196" s="4"/>
-      <c r="F196" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="G196" s="4"/>
-      <c r="H196" s="4"/>
-      <c r="I196" s="4"/>
-      <c r="J196" s="4"/>
-      <c r="K196" s="4"/>
-    </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A197" s="4"/>
-      <c r="B197" s="4"/>
-      <c r="C197" s="4"/>
-      <c r="D197" s="4"/>
-      <c r="E197" s="4"/>
-      <c r="F197" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="G197" s="4"/>
-      <c r="H197" s="4"/>
-      <c r="I197" s="4"/>
-      <c r="J197" s="4"/>
-      <c r="K197" s="4"/>
-    </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A198" s="4"/>
-      <c r="B198" s="4"/>
-      <c r="C198" s="4"/>
-      <c r="D198" s="4"/>
-      <c r="E198" s="4"/>
-      <c r="F198" s="4" t="s">
-        <v>196</v>
-      </c>
-      <c r="G198" s="4"/>
-      <c r="H198" s="4"/>
-      <c r="I198" s="4"/>
-      <c r="J198" s="4"/>
-      <c r="K198" s="4"/>
-    </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A199" s="4"/>
-      <c r="B199" s="4"/>
-      <c r="C199" s="4"/>
-      <c r="D199" s="4"/>
-      <c r="E199" s="4"/>
-      <c r="F199" s="4" t="s">
-        <v>194</v>
-      </c>
-      <c r="G199" s="4"/>
-      <c r="H199" s="4"/>
-      <c r="I199" s="4"/>
-      <c r="J199" s="4"/>
-      <c r="K199" s="4"/>
-    </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A200" s="4"/>
-      <c r="B200" s="4"/>
-      <c r="C200" s="4"/>
-      <c r="D200" s="4"/>
-      <c r="E200" s="4"/>
-      <c r="F200" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="G200" s="4"/>
-      <c r="H200" s="4"/>
-      <c r="I200" s="4"/>
-      <c r="J200" s="4"/>
-      <c r="K200" s="4"/>
-    </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A201" s="4"/>
-      <c r="B201" s="4"/>
-      <c r="C201" s="4"/>
-      <c r="D201" s="4"/>
-      <c r="E201" s="4"/>
-      <c r="F201" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="G201" s="4"/>
-      <c r="H201" s="4"/>
-      <c r="I201" s="4"/>
-      <c r="J201" s="4"/>
-      <c r="K201" s="4"/>
-    </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A202" s="4"/>
-      <c r="B202" s="4"/>
-      <c r="C202" s="4"/>
-      <c r="D202" s="4"/>
-      <c r="E202" s="4"/>
-      <c r="F202" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="G202" s="4"/>
-      <c r="H202" s="4"/>
-      <c r="I202" s="4"/>
-      <c r="J202" s="4"/>
-      <c r="K202" s="4"/>
-    </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A203" s="4"/>
-      <c r="B203" s="4"/>
-      <c r="C203" s="4"/>
-      <c r="D203" s="4"/>
-      <c r="E203" s="4"/>
-      <c r="F203" s="4" t="s">
-        <v>200</v>
-      </c>
-      <c r="G203" s="4"/>
-      <c r="H203" s="4"/>
-      <c r="I203" s="4"/>
-      <c r="J203" s="4"/>
-      <c r="K203" s="4"/>
-    </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A204" s="4"/>
-      <c r="B204" s="4"/>
-      <c r="C204" s="4"/>
-      <c r="D204" s="4"/>
-      <c r="E204" s="4"/>
-      <c r="F204" s="4" t="s">
-        <v>201</v>
-      </c>
-      <c r="G204" s="4"/>
-      <c r="H204" s="4"/>
-      <c r="I204" s="4"/>
-      <c r="J204" s="4"/>
-      <c r="K204" s="4"/>
-    </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A205" s="4"/>
-      <c r="B205" s="4"/>
-      <c r="C205" s="4"/>
-      <c r="D205" s="4"/>
-      <c r="E205" s="4"/>
-      <c r="F205" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="G205" s="4"/>
-      <c r="H205" s="4"/>
-      <c r="I205" s="4"/>
-      <c r="J205" s="4"/>
-      <c r="K205" s="4"/>
-    </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A206" s="4"/>
-      <c r="B206" s="4"/>
-      <c r="C206" s="4"/>
-      <c r="D206" s="4"/>
-      <c r="E206" s="4"/>
-      <c r="F206" s="4"/>
-      <c r="G206" s="4"/>
-      <c r="H206" s="4"/>
-      <c r="I206" s="4"/>
-      <c r="J206" s="4"/>
-      <c r="K206" s="4"/>
-    </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A207" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B207" s="4"/>
-      <c r="C207" s="4"/>
-      <c r="D207" s="4"/>
-      <c r="E207" s="4"/>
-      <c r="F207" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="G207" s="4"/>
-      <c r="H207" s="4"/>
-      <c r="I207" s="4"/>
-      <c r="J207" s="4"/>
-      <c r="K207" s="4"/>
-    </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A208" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="B208" s="4"/>
-      <c r="C208" s="4"/>
-      <c r="D208" s="4"/>
-      <c r="E208" s="4"/>
-      <c r="F208" s="4" t="s">
-        <v>242</v>
-      </c>
-      <c r="G208" s="4"/>
-      <c r="H208" s="4"/>
-      <c r="I208" s="4"/>
-      <c r="J208" s="4"/>
-      <c r="K208" s="4"/>
-    </row>
-    <row r="209" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A209" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="B209" s="4"/>
-      <c r="C209" s="4"/>
-      <c r="D209" s="4"/>
-      <c r="E209" s="4"/>
-      <c r="F209" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="G209" s="4"/>
-      <c r="H209" s="4"/>
-      <c r="I209" s="4"/>
-      <c r="J209" s="4"/>
-      <c r="K209" s="4"/>
-    </row>
-    <row r="210" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A210" s="4"/>
-      <c r="B210" s="4"/>
-      <c r="C210" s="4"/>
-      <c r="D210" s="4"/>
-      <c r="E210" s="4"/>
-      <c r="F210" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="G210" s="4"/>
-      <c r="H210" s="4"/>
-      <c r="I210" s="4"/>
-      <c r="J210" s="4"/>
-      <c r="K210" s="4"/>
-    </row>
-    <row r="211" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A211" s="4"/>
-      <c r="B211" s="4"/>
-      <c r="C211" s="4"/>
-      <c r="D211" s="4"/>
-      <c r="E211" s="4"/>
-      <c r="F211" s="4" t="s">
-        <v>208</v>
-      </c>
-      <c r="G211" s="4"/>
-      <c r="H211" s="4"/>
-      <c r="I211" s="4"/>
-      <c r="J211" s="4"/>
-      <c r="K211" s="4"/>
-    </row>
-    <row r="212" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A212" s="4"/>
-      <c r="B212" s="4"/>
-      <c r="C212" s="4"/>
-      <c r="D212" s="4"/>
-      <c r="E212" s="4"/>
-      <c r="F212" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="G212" s="4"/>
-      <c r="H212" s="4"/>
-      <c r="I212" s="4"/>
-      <c r="J212" s="4"/>
-      <c r="K212" s="4"/>
-    </row>
-    <row r="213" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A213" s="4"/>
       <c r="B213" s="4"/>
       <c r="C213" s="4"/>
       <c r="D213" s="4"/>
       <c r="E213" s="4"/>
       <c r="F213" s="4" t="s">
-        <v>210</v>
+        <v>191</v>
       </c>
       <c r="G213" s="4"/>
       <c r="H213" s="4"/>
@@ -4386,13 +4328,15 @@
       <c r="K213" s="4"/>
     </row>
     <row r="214" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A214" s="4"/>
+      <c r="A214" s="4" t="s">
+        <v>164</v>
+      </c>
       <c r="B214" s="4"/>
       <c r="C214" s="4"/>
       <c r="D214" s="4"/>
       <c r="E214" s="4"/>
       <c r="F214" s="4" t="s">
-        <v>211</v>
+        <v>227</v>
       </c>
       <c r="G214" s="4"/>
       <c r="H214" s="4"/>
@@ -4401,13 +4345,15 @@
       <c r="K214" s="4"/>
     </row>
     <row r="215" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A215" s="4"/>
+      <c r="A215" s="4" t="s">
+        <v>160</v>
+      </c>
       <c r="B215" s="4"/>
       <c r="C215" s="4"/>
       <c r="D215" s="4"/>
       <c r="E215" s="4"/>
       <c r="F215" s="4" t="s">
-        <v>212</v>
+        <v>168</v>
       </c>
       <c r="G215" s="4"/>
       <c r="H215" s="4"/>
@@ -4422,7 +4368,7 @@
       <c r="D216" s="4"/>
       <c r="E216" s="4"/>
       <c r="F216" s="4" t="s">
-        <v>213</v>
+        <v>176</v>
       </c>
       <c r="G216" s="4"/>
       <c r="H216" s="4"/>
@@ -4437,7 +4383,7 @@
       <c r="D217" s="4"/>
       <c r="E217" s="4"/>
       <c r="F217" s="4" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="G217" s="4"/>
       <c r="H217" s="4"/>
@@ -4452,7 +4398,7 @@
       <c r="D218" s="4"/>
       <c r="E218" s="4"/>
       <c r="F218" s="4" t="s">
-        <v>215</v>
+        <v>228</v>
       </c>
       <c r="G218" s="4"/>
       <c r="H218" s="4"/>
@@ -4467,7 +4413,7 @@
       <c r="D219" s="4"/>
       <c r="E219" s="4"/>
       <c r="F219" s="4" t="s">
-        <v>216</v>
+        <v>229</v>
       </c>
       <c r="G219" s="4"/>
       <c r="H219" s="4"/>
@@ -4481,7 +4427,9 @@
       <c r="C220" s="4"/>
       <c r="D220" s="4"/>
       <c r="E220" s="4"/>
-      <c r="F220" s="4"/>
+      <c r="F220" s="4" t="s">
+        <v>230</v>
+      </c>
       <c r="G220" s="4"/>
       <c r="H220" s="4"/>
       <c r="I220" s="4"/>
@@ -4489,15 +4437,13 @@
       <c r="K220" s="4"/>
     </row>
     <row r="221" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A221" s="4" t="s">
-        <v>0</v>
-      </c>
+      <c r="A221" s="4"/>
       <c r="B221" s="4"/>
       <c r="C221" s="4"/>
       <c r="D221" s="4"/>
       <c r="E221" s="4"/>
       <c r="F221" s="4" t="s">
-        <v>244</v>
+        <v>231</v>
       </c>
       <c r="G221" s="4"/>
       <c r="H221" s="4"/>
@@ -4506,16 +4452,12 @@
       <c r="K221" s="4"/>
     </row>
     <row r="222" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A222" s="4" t="s">
-        <v>205</v>
-      </c>
+      <c r="A222" s="4"/>
       <c r="B222" s="4"/>
       <c r="C222" s="4"/>
       <c r="D222" s="4"/>
       <c r="E222" s="4"/>
-      <c r="F222" s="4" t="s">
-        <v>245</v>
-      </c>
+      <c r="F222" s="4"/>
       <c r="G222" s="4"/>
       <c r="H222" s="4"/>
       <c r="I222" s="4"/>
@@ -4524,14 +4466,14 @@
     </row>
     <row r="223" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A223" s="4" t="s">
-        <v>238</v>
+        <v>0</v>
       </c>
       <c r="B223" s="4"/>
       <c r="C223" s="4"/>
       <c r="D223" s="4"/>
       <c r="E223" s="4"/>
       <c r="F223" s="4" t="s">
-        <v>246</v>
+        <v>225</v>
       </c>
       <c r="G223" s="4"/>
       <c r="H223" s="4"/>
@@ -4540,13 +4482,15 @@
       <c r="K223" s="4"/>
     </row>
     <row r="224" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A224" s="4"/>
+      <c r="A224" s="4" t="s">
+        <v>161</v>
+      </c>
       <c r="B224" s="4"/>
       <c r="C224" s="4"/>
       <c r="D224" s="4"/>
       <c r="E224" s="4"/>
       <c r="F224" s="4" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="G224" s="4"/>
       <c r="H224" s="4"/>
@@ -4555,13 +4499,15 @@
       <c r="K224" s="4"/>
     </row>
     <row r="225" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A225" s="4"/>
+      <c r="A225" s="4" t="s">
+        <v>165</v>
+      </c>
       <c r="B225" s="4"/>
       <c r="C225" s="4"/>
       <c r="D225" s="4"/>
       <c r="E225" s="4"/>
       <c r="F225" s="4" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="G225" s="4"/>
       <c r="H225" s="4"/>
@@ -4576,7 +4522,7 @@
       <c r="D226" s="4"/>
       <c r="E226" s="4"/>
       <c r="F226" s="4" t="s">
-        <v>219</v>
+        <v>116</v>
       </c>
       <c r="G226" s="4"/>
       <c r="H226" s="4"/>
@@ -4591,7 +4537,7 @@
       <c r="D227" s="4"/>
       <c r="E227" s="4"/>
       <c r="F227" s="4" t="s">
-        <v>220</v>
+        <v>192</v>
       </c>
       <c r="G227" s="4"/>
       <c r="H227" s="4"/>
@@ -4606,7 +4552,7 @@
       <c r="D228" s="4"/>
       <c r="E228" s="4"/>
       <c r="F228" s="4" t="s">
-        <v>221</v>
+        <v>249</v>
       </c>
       <c r="G228" s="4"/>
       <c r="H228" s="4"/>
@@ -4621,7 +4567,7 @@
       <c r="D229" s="4"/>
       <c r="E229" s="4"/>
       <c r="F229" s="4" t="s">
-        <v>222</v>
+        <v>250</v>
       </c>
       <c r="G229" s="4"/>
       <c r="H229" s="4"/>
@@ -4636,7 +4582,7 @@
       <c r="D230" s="4"/>
       <c r="E230" s="4"/>
       <c r="F230" s="4" t="s">
-        <v>223</v>
+        <v>251</v>
       </c>
       <c r="G230" s="4"/>
       <c r="H230" s="4"/>
@@ -4651,7 +4597,7 @@
       <c r="D231" s="4"/>
       <c r="E231" s="4"/>
       <c r="F231" s="4" t="s">
-        <v>224</v>
+        <v>252</v>
       </c>
       <c r="G231" s="4"/>
       <c r="H231" s="4"/>
@@ -4665,9 +4611,7 @@
       <c r="C232" s="4"/>
       <c r="D232" s="4"/>
       <c r="E232" s="4"/>
-      <c r="F232" s="4" t="s">
-        <v>225</v>
-      </c>
+      <c r="F232" s="4"/>
       <c r="G232" s="4"/>
       <c r="H232" s="4"/>
       <c r="I232" s="4"/>
@@ -4675,13 +4619,15 @@
       <c r="K232" s="4"/>
     </row>
     <row r="233" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A233" s="4"/>
+      <c r="A233" s="4" t="s">
+        <v>0</v>
+      </c>
       <c r="B233" s="4"/>
       <c r="C233" s="4"/>
       <c r="D233" s="4"/>
       <c r="E233" s="4"/>
       <c r="F233" s="4" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="G233" s="4"/>
       <c r="H233" s="4"/>
@@ -4690,12 +4636,16 @@
       <c r="K233" s="4"/>
     </row>
     <row r="234" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A234" s="4"/>
+      <c r="A234" s="4" t="s">
+        <v>163</v>
+      </c>
       <c r="B234" s="4"/>
       <c r="C234" s="4"/>
       <c r="D234" s="4"/>
       <c r="E234" s="4"/>
-      <c r="F234" s="4"/>
+      <c r="F234" s="4" t="s">
+        <v>234</v>
+      </c>
       <c r="G234" s="4"/>
       <c r="H234" s="4"/>
       <c r="I234" s="4"/>
@@ -4704,14 +4654,14 @@
     </row>
     <row r="235" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A235" s="4" t="s">
-        <v>0</v>
+        <v>166</v>
       </c>
       <c r="B235" s="4"/>
       <c r="C235" s="4"/>
       <c r="D235" s="4"/>
       <c r="E235" s="4"/>
       <c r="F235" s="4" t="s">
-        <v>247</v>
+        <v>235</v>
       </c>
       <c r="G235" s="4"/>
       <c r="H235" s="4"/>
@@ -4720,15 +4670,13 @@
       <c r="K235" s="4"/>
     </row>
     <row r="236" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A236" s="4" t="s">
-        <v>204</v>
-      </c>
+      <c r="A236" s="4"/>
       <c r="B236" s="4"/>
       <c r="C236" s="4"/>
       <c r="D236" s="4"/>
       <c r="E236" s="4"/>
       <c r="F236" s="4" t="s">
-        <v>248</v>
+        <v>120</v>
       </c>
       <c r="G236" s="4"/>
       <c r="H236" s="4"/>
@@ -4737,15 +4685,13 @@
       <c r="K236" s="4"/>
     </row>
     <row r="237" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A237" s="4" t="s">
-        <v>239</v>
-      </c>
+      <c r="A237" s="4"/>
       <c r="B237" s="4"/>
       <c r="C237" s="4"/>
       <c r="D237" s="4"/>
       <c r="E237" s="4"/>
       <c r="F237" s="4" t="s">
-        <v>249</v>
+        <v>218</v>
       </c>
       <c r="G237" s="4"/>
       <c r="H237" s="4"/>
@@ -4760,7 +4706,7 @@
       <c r="D238" s="4"/>
       <c r="E238" s="4"/>
       <c r="F238" s="4" t="s">
-        <v>227</v>
+        <v>236</v>
       </c>
       <c r="G238" s="4"/>
       <c r="H238" s="4"/>
@@ -4775,7 +4721,7 @@
       <c r="D239" s="4"/>
       <c r="E239" s="4"/>
       <c r="F239" s="4" t="s">
-        <v>228</v>
+        <v>237</v>
       </c>
       <c r="G239" s="4"/>
       <c r="H239" s="4"/>
@@ -4790,7 +4736,7 @@
       <c r="D240" s="4"/>
       <c r="E240" s="4"/>
       <c r="F240" s="4" t="s">
-        <v>229</v>
+        <v>238</v>
       </c>
       <c r="G240" s="4"/>
       <c r="H240" s="4"/>
@@ -4805,7 +4751,7 @@
       <c r="D241" s="4"/>
       <c r="E241" s="4"/>
       <c r="F241" s="4" t="s">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="G241" s="4"/>
       <c r="H241" s="4"/>
@@ -4819,9 +4765,7 @@
       <c r="C242" s="4"/>
       <c r="D242" s="4"/>
       <c r="E242" s="4"/>
-      <c r="F242" s="4" t="s">
-        <v>231</v>
-      </c>
+      <c r="F242" s="4"/>
       <c r="G242" s="4"/>
       <c r="H242" s="4"/>
       <c r="I242" s="4"/>
@@ -4829,13 +4773,15 @@
       <c r="K242" s="4"/>
     </row>
     <row r="243" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A243" s="4"/>
+      <c r="A243" s="4" t="s">
+        <v>0</v>
+      </c>
       <c r="B243" s="4"/>
       <c r="C243" s="4"/>
       <c r="D243" s="4"/>
       <c r="E243" s="4"/>
       <c r="F243" s="4" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="G243" s="4"/>
       <c r="H243" s="4"/>
@@ -4844,13 +4790,15 @@
       <c r="K243" s="4"/>
     </row>
     <row r="244" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A244" s="4"/>
+      <c r="A244" s="4" t="s">
+        <v>162</v>
+      </c>
       <c r="B244" s="4"/>
       <c r="C244" s="4"/>
       <c r="D244" s="4"/>
       <c r="E244" s="4"/>
       <c r="F244" s="4" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="G244" s="4"/>
       <c r="H244" s="4"/>
@@ -4859,13 +4807,15 @@
       <c r="K244" s="4"/>
     </row>
     <row r="245" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A245" s="4"/>
+      <c r="A245" s="4" t="s">
+        <v>167</v>
+      </c>
       <c r="B245" s="4"/>
       <c r="C245" s="4"/>
       <c r="D245" s="4"/>
       <c r="E245" s="4"/>
       <c r="F245" s="4" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="G245" s="4"/>
       <c r="H245" s="4"/>
@@ -4880,7 +4830,7 @@
       <c r="D246" s="4"/>
       <c r="E246" s="4"/>
       <c r="F246" s="4" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="G246" s="4"/>
       <c r="H246" s="4"/>
@@ -4895,7 +4845,7 @@
       <c r="D247" s="4"/>
       <c r="E247" s="4"/>
       <c r="F247" s="4" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="G247" s="4"/>
       <c r="H247" s="4"/>
@@ -4903,6 +4853,66 @@
       <c r="J247" s="4"/>
       <c r="K247" s="4"/>
     </row>
+    <row r="248" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A248" s="4"/>
+      <c r="B248" s="4"/>
+      <c r="C248" s="4"/>
+      <c r="D248" s="4"/>
+      <c r="E248" s="4"/>
+      <c r="F248" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="G248" s="4"/>
+      <c r="H248" s="4"/>
+      <c r="I248" s="4"/>
+      <c r="J248" s="4"/>
+      <c r="K248" s="4"/>
+    </row>
+    <row r="249" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A249" s="4"/>
+      <c r="B249" s="4"/>
+      <c r="C249" s="4"/>
+      <c r="D249" s="4"/>
+      <c r="E249" s="4"/>
+      <c r="F249" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="G249" s="4"/>
+      <c r="H249" s="4"/>
+      <c r="I249" s="4"/>
+      <c r="J249" s="4"/>
+      <c r="K249" s="4"/>
+    </row>
+    <row r="250" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A250" s="4"/>
+      <c r="B250" s="4"/>
+      <c r="C250" s="4"/>
+      <c r="D250" s="4"/>
+      <c r="E250" s="4"/>
+      <c r="F250" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="G250" s="4"/>
+      <c r="H250" s="4"/>
+      <c r="I250" s="4"/>
+      <c r="J250" s="4"/>
+      <c r="K250" s="4"/>
+    </row>
+    <row r="251" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A251" s="4"/>
+      <c r="B251" s="4"/>
+      <c r="C251" s="4"/>
+      <c r="D251" s="4"/>
+      <c r="E251" s="4"/>
+      <c r="F251" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="G251" s="4"/>
+      <c r="H251" s="4"/>
+      <c r="I251" s="4"/>
+      <c r="J251" s="4"/>
+      <c r="K251" s="4"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Payments service and AWS S3 Bucket connections added to architecture diagram
</commit_message>
<xml_diff>
--- a/DBMS Game Store Docs/User Stories.xlsx
+++ b/DBMS Game Store Docs/User Stories.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ryanc\Desktop\final_year_project\DBMS Game Store Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518A0D7B-13FE-4149-B0D8-078C870DFE1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D03F2BC8-9806-4DDB-8FB0-FD3B06323398}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="0" windowWidth="13410" windowHeight="16305" xr2:uid="{91133E6D-6CC4-4AFD-BF36-5C9837FF4593}"/>
+    <workbookView xWindow="15015" yWindow="1245" windowWidth="12510" windowHeight="12750" xr2:uid="{91133E6D-6CC4-4AFD-BF36-5C9837FF4593}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -890,7 +890,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -902,7 +902,6 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1237,7 +1236,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62F77FC3-F402-4BE8-8A68-6767566B15A6}">
-  <dimension ref="A1:O251"/>
+  <dimension ref="A1:K251"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
@@ -3118,7 +3117,7 @@
       <c r="J128" s="3"/>
       <c r="K128" s="3"/>
     </row>
-    <row r="129" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
@@ -3133,7 +3132,7 @@
       <c r="J129" s="3"/>
       <c r="K129" s="3"/>
     </row>
-    <row r="130" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
@@ -3148,7 +3147,7 @@
       <c r="J130" s="3"/>
       <c r="K130" s="3"/>
     </row>
-    <row r="131" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
@@ -3163,7 +3162,7 @@
       <c r="J131" s="3"/>
       <c r="K131" s="3"/>
     </row>
-    <row r="132" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
@@ -3178,7 +3177,7 @@
       <c r="J132" s="3"/>
       <c r="K132" s="3"/>
     </row>
-    <row r="133" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
@@ -3193,7 +3192,7 @@
       <c r="J133" s="3"/>
       <c r="K133" s="3"/>
     </row>
-    <row r="134" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
@@ -3208,7 +3207,7 @@
       <c r="J134" s="3"/>
       <c r="K134" s="3"/>
     </row>
-    <row r="135" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
@@ -3221,7 +3220,7 @@
       <c r="J135" s="3"/>
       <c r="K135" s="3"/>
     </row>
-    <row r="136" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A136" s="3" t="s">
         <v>80</v>
       </c>
@@ -3238,7 +3237,7 @@
       <c r="J136" s="3"/>
       <c r="K136" s="3"/>
     </row>
-    <row r="137" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A137" s="3" t="s">
         <v>59</v>
       </c>
@@ -3255,7 +3254,7 @@
       <c r="J137" s="3"/>
       <c r="K137" s="3"/>
     </row>
-    <row r="138" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A138" s="3" t="s">
         <v>21</v>
       </c>
@@ -3272,7 +3271,7 @@
       <c r="J138" s="3"/>
       <c r="K138" s="3"/>
     </row>
-    <row r="139" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
@@ -3287,7 +3286,7 @@
       <c r="J139" s="3"/>
       <c r="K139" s="3"/>
     </row>
-    <row r="140" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
@@ -3302,7 +3301,7 @@
       <c r="J140" s="3"/>
       <c r="K140" s="3"/>
     </row>
-    <row r="141" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
@@ -3317,7 +3316,7 @@
       <c r="J141" s="3"/>
       <c r="K141" s="3"/>
     </row>
-    <row r="142" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
@@ -3331,12 +3330,8 @@
       <c r="I142" s="3"/>
       <c r="J142" s="3"/>
       <c r="K142" s="3"/>
-      <c r="L142" s="11"/>
-      <c r="M142" s="11"/>
-      <c r="N142" s="11"/>
-      <c r="O142" s="11"/>
-    </row>
-    <row r="143" spans="1:15" x14ac:dyDescent="0.25">
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
@@ -3351,7 +3346,7 @@
       <c r="J143" s="3"/>
       <c r="K143" s="3"/>
     </row>
-    <row r="144" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A144" s="3"/>
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>

</xml_diff>